<commit_message>
Update FeedMgmt to remove feed_par_DM
</commit_message>
<xml_diff>
--- a/mini/data/default/FeedMgmt.xlsx
+++ b/mini/data/default/FeedMgmt.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="91">
   <si>
     <t xml:space="preserve">Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -327,12 +327,6 @@
   </si>
   <si>
     <t xml:space="preserve">General</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feed_par_DM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg DM/kg as fed</t>
   </si>
   <si>
     <t xml:space="preserve">GE</t>
@@ -517,80 +511,72 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -847,22 +833,22 @@
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -882,103 +868,103 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:S128"/>
+  <dimension ref="A1:S1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="20.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="19.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="9.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="10.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="38.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="38.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="R2" s="3"/>
-      <c r="S2" s="5"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N3" s="6" t="s">
@@ -1002,13 +988,13 @@
       <c r="Q4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N5" s="0" t="s">
+      <c r="N5" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O5" s="9" t="n">
@@ -1016,13 +1002,13 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N6" s="0" t="s">
+      <c r="N6" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O6" s="9" t="n">
@@ -1030,13 +1016,13 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="I7" s="0" t="s">
+      <c r="I7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N7" s="0" t="s">
+      <c r="N7" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O7" s="9" t="n">
@@ -1044,13 +1030,13 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="0" t="s">
+      <c r="I8" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N8" s="0" t="s">
+      <c r="N8" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O8" s="9" t="n">
@@ -1075,13 +1061,13 @@
       <c r="Q9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F10" s="0" t="s">
+      <c r="F10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J10" s="0" t="s">
+      <c r="J10" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="N10" s="0" t="s">
+      <c r="N10" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O10" s="9" t="n">
@@ -1089,13 +1075,13 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J11" s="0" t="s">
+      <c r="J11" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="N11" s="0" t="s">
+      <c r="N11" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O11" s="9" t="n">
@@ -1103,13 +1089,13 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="J12" s="0" t="s">
+      <c r="J12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="N12" s="0" t="s">
+      <c r="N12" s="1" t="s">
         <v>25</v>
       </c>
       <c r="O12" s="9" t="n">
@@ -1129,34 +1115,34 @@
       <c r="O15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
-    </row>
-    <row r="17" s="5" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+      <c r="N16" s="4"/>
+      <c r="O16" s="4"/>
+      <c r="P16" s="4"/>
+      <c r="Q16" s="4"/>
+      <c r="R16" s="4"/>
+    </row>
+    <row r="17" s="1" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N18" s="6" t="s">
@@ -1173,30 +1159,30 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I19" s="0" t="s">
+      <c r="I19" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N19" s="0" t="s">
+      <c r="N19" s="1" t="s">
         <v>41</v>
       </c>
       <c r="O19" s="11" t="n">
         <v>95</v>
       </c>
-      <c r="P19" s="0" t="s">
+      <c r="P19" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I20" s="0" t="s">
+      <c r="I20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N20" s="0" t="s">
+      <c r="N20" s="1" t="s">
         <v>41</v>
       </c>
       <c r="O20" s="11" t="n">
         <v>95</v>
       </c>
-      <c r="P20" s="0" t="s">
+      <c r="P20" s="1" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1205,38 +1191,38 @@
       <c r="Q21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+      <c r="A22" s="12" t="s">
         <v>43</v>
       </c>
       <c r="O22" s="11"/>
       <c r="Q22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I23" s="0" t="s">
+      <c r="I23" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="N23" s="0" t="s">
+      <c r="N23" s="1" t="s">
         <v>44</v>
       </c>
       <c r="O23" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="P23" s="0" t="s">
+      <c r="P23" s="1" t="s">
         <v>42</v>
       </c>
       <c r="Q23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I24" s="0" t="s">
+      <c r="I24" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N24" s="0" t="s">
+      <c r="N24" s="1" t="s">
         <v>44</v>
       </c>
       <c r="O24" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="P24" s="0" t="s">
+      <c r="P24" s="1" t="s">
         <v>42</v>
       </c>
       <c r="Q24" s="11"/>
@@ -1246,26 +1232,26 @@
       <c r="Q25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="O26" s="3"/>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
+      <c r="K26" s="4"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="4"/>
+      <c r="O26" s="4"/>
+      <c r="P26" s="4"/>
+      <c r="Q26" s="4"/>
+      <c r="R26" s="4"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N27" s="6" t="s">
@@ -1282,71 +1268,71 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-      <c r="M28" s="3"/>
-      <c r="N28" s="3"/>
-      <c r="O28" s="3"/>
-      <c r="P28" s="3"/>
-      <c r="Q28" s="3"/>
-      <c r="R28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+      <c r="O28" s="4"/>
+      <c r="P28" s="4"/>
+      <c r="Q28" s="4"/>
+      <c r="R28" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="H30" s="0" t="s">
+      <c r="A30" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H30" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I30" s="0" t="s">
+      <c r="I30" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N30" s="0" t="s">
+      <c r="N30" s="1" t="s">
         <v>50</v>
       </c>
       <c r="O30" s="10" t="n">
         <v>30</v>
       </c>
-      <c r="P30" s="0" t="s">
+      <c r="P30" s="1" t="s">
         <v>42</v>
       </c>
       <c r="Q30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="0" t="s">
+      <c r="A31" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E31" s="0" t="s">
+      <c r="E31" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H31" s="0" t="s">
+      <c r="H31" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="I31" s="0" t="s">
+      <c r="I31" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N31" s="0" t="s">
+      <c r="N31" s="1" t="s">
         <v>50</v>
       </c>
       <c r="O31" s="10" t="n">
         <v>10</v>
       </c>
-      <c r="P31" s="0" t="s">
+      <c r="P31" s="1" t="s">
         <v>42</v>
       </c>
       <c r="Q31" s="10"/>
@@ -1356,26 +1342,26 @@
       <c r="Q32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-      <c r="I33" s="3"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="3"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="3"/>
-      <c r="O33" s="3"/>
-      <c r="P33" s="3"/>
-      <c r="Q33" s="3"/>
-      <c r="R33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
+      <c r="K33" s="4"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="4"/>
+      <c r="O33" s="4"/>
+      <c r="P33" s="4"/>
+      <c r="Q33" s="4"/>
+      <c r="R33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N34" s="6" t="s">
@@ -1406,16 +1392,16 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="0" t="s">
+      <c r="A36" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="E36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G36" s="0" t="s">
+      <c r="G36" s="1" t="s">
         <v>56</v>
       </c>
       <c r="N36" s="10" t="s">
@@ -1431,15 +1417,15 @@
       <c r="Q36" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="R36" s="0" t="s">
+      <c r="R36" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="G37" s="0" t="s">
+      <c r="A37" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>56</v>
       </c>
       <c r="N37" s="10" t="s">
@@ -1455,7 +1441,7 @@
       <c r="Q37" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="R37" s="0" t="s">
+      <c r="R37" s="1" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1466,16 +1452,16 @@
       <c r="Q38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="0" t="s">
+      <c r="A39" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="E39" s="0" t="s">
+      <c r="E39" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="G39" s="1" t="s">
         <v>56</v>
       </c>
       <c r="N39" s="10" t="s">
@@ -1490,18 +1476,18 @@
       <c r="Q39" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="R39" s="0" t="s">
+      <c r="R39" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="E40" s="0" t="s">
+      <c r="A40" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E40" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G40" s="0" t="s">
+      <c r="G40" s="1" t="s">
         <v>56</v>
       </c>
       <c r="N40" s="10" t="s">
@@ -1516,15 +1502,15 @@
       <c r="Q40" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="R40" s="0" t="s">
+      <c r="R40" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="G41" s="0" t="s">
+      <c r="A41" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G41" s="1" t="s">
         <v>56</v>
       </c>
       <c r="N41" s="10" t="s">
@@ -1540,7 +1526,7 @@
       <c r="Q41" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="R41" s="0" t="s">
+      <c r="R41" s="1" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1552,7 +1538,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11"/>
-      <c r="G43" s="0" t="s">
+      <c r="G43" s="1" t="s">
         <v>63</v>
       </c>
       <c r="N43" s="10" t="s">
@@ -1565,7 +1551,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="11"/>
-      <c r="G44" s="0" t="s">
+      <c r="G44" s="1" t="s">
         <v>63</v>
       </c>
       <c r="N44" s="10" t="s">
@@ -1580,7 +1566,7 @@
       <c r="Q44" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="R44" s="0" t="s">
+      <c r="R44" s="1" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1592,29 +1578,29 @@
       <c r="Q45" s="11"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="2" t="s">
+      <c r="A46" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-      <c r="G46" s="3"/>
-      <c r="H46" s="3"/>
-      <c r="I46" s="3"/>
-      <c r="J46" s="3"/>
-      <c r="K46" s="3"/>
-      <c r="L46" s="3"/>
-      <c r="M46" s="3"/>
-      <c r="N46" s="3"/>
-      <c r="O46" s="3"/>
-      <c r="P46" s="3"/>
-      <c r="Q46" s="3"/>
-      <c r="R46" s="3"/>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="4"/>
+      <c r="J46" s="4"/>
+      <c r="K46" s="4"/>
+      <c r="L46" s="4"/>
+      <c r="M46" s="4"/>
+      <c r="N46" s="4"/>
+      <c r="O46" s="4"/>
+      <c r="P46" s="4"/>
+      <c r="Q46" s="4"/>
+      <c r="R46" s="4"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="A47" s="1" t="s">
         <v>48</v>
       </c>
       <c r="O47" s="10"/>
@@ -1627,7 +1613,7 @@
       <c r="Q48" s="11"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N49" s="0" t="s">
+      <c r="N49" s="1" t="s">
         <v>69</v>
       </c>
       <c r="O49" s="10" t="n">
@@ -1646,28 +1632,28 @@
       <c r="Q50" s="11"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2" t="s">
+      <c r="A51" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="3"/>
-      <c r="F51" s="3"/>
-      <c r="G51" s="3"/>
-      <c r="H51" s="3"/>
-      <c r="I51" s="3"/>
-      <c r="J51" s="3"/>
-      <c r="K51" s="3"/>
-      <c r="L51" s="3"/>
-      <c r="M51" s="3"/>
-      <c r="N51" s="3"/>
-      <c r="O51" s="3"/>
-      <c r="P51" s="3"/>
-      <c r="Q51" s="3" t="s">
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="4"/>
+      <c r="F51" s="4"/>
+      <c r="G51" s="4"/>
+      <c r="H51" s="4"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
+      <c r="K51" s="4"/>
+      <c r="L51" s="4"/>
+      <c r="M51" s="4"/>
+      <c r="N51" s="4"/>
+      <c r="O51" s="4"/>
+      <c r="P51" s="4"/>
+      <c r="Q51" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="R51" s="3"/>
+      <c r="R51" s="4"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
@@ -1675,1018 +1661,940 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F53" s="0" t="s">
+      <c r="F53" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="N53" s="0" t="s">
+      <c r="M53" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O53" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="P53" s="0" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q53" s="11"/>
+      <c r="N53" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O53" s="13" t="n">
+        <v>17.3169484</v>
+      </c>
+      <c r="P53" s="1" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F54" s="0" t="s">
+      <c r="F54" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N54" s="0" t="s">
+      <c r="M54" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O54" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="Q54" s="11"/>
+      <c r="N54" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O54" s="13" t="n">
+        <v>17.150216</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F55" s="0" t="s">
+      <c r="F55" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="N55" s="0" t="s">
+      <c r="M55" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O55" s="15" t="n">
-        <v>100</v>
+      <c r="N55" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O55" s="13" t="n">
+        <v>17.41143707</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F56" s="0" t="s">
+      <c r="F56" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="N56" s="0" t="s">
+      <c r="M56" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O56" s="15" t="n">
-        <v>86</v>
+      <c r="N56" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O56" s="13" t="n">
+        <v>18.2100232</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F57" s="0" t="s">
+      <c r="F57" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="N57" s="0" t="s">
+      <c r="M57" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O57" s="15" t="n">
-        <v>87.5</v>
+      <c r="N57" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O57" s="13" t="n">
+        <v>19.589488</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F58" s="0" t="s">
+      <c r="F58" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="N58" s="0" t="s">
+      <c r="M58" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O58" s="15" t="n">
-        <v>89.5</v>
-      </c>
-      <c r="Q58" s="11"/>
+      <c r="N58" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O58" s="13" t="n">
+        <v>19.4920008</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F59" s="0" t="s">
+      <c r="F59" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="N59" s="0" t="s">
+      <c r="M59" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="O59" s="15" t="n">
-        <v>87</v>
+      <c r="N59" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O59" s="13" t="n">
+        <v>18.194124</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O60" s="15"/>
+      <c r="O60" s="13"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F61" s="0" t="s">
+      <c r="F61" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M61" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N61" s="0" t="s">
+      <c r="M61" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N61" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O61" s="15" t="n">
-        <v>17.3169484</v>
-      </c>
-      <c r="P61" s="0" t="s">
-        <v>79</v>
+        <v>7.55</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F62" s="0" t="s">
+      <c r="F62" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M62" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N62" s="0" t="s">
+      <c r="M62" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N62" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O62" s="15" t="n">
-        <v>17.150216</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F63" s="0" t="s">
+      <c r="F63" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M63" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N63" s="0" t="s">
+      <c r="M63" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N63" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O63" s="15" t="n">
-        <v>17.41143707</v>
+        <v>6.566666667</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F64" s="0" t="s">
+      <c r="F64" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M64" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N64" s="0" t="s">
+      <c r="M64" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N64" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O64" s="15" t="n">
-        <v>18.2100232</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F65" s="0" t="s">
+      <c r="F65" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M65" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N65" s="0" t="s">
+      <c r="M65" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N65" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O65" s="15" t="n">
-        <v>19.589488</v>
+        <v>7.15</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F66" s="0" t="s">
+      <c r="F66" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M66" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N66" s="0" t="s">
+      <c r="M66" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N66" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O66" s="15" t="n">
-        <v>19.4920008</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F67" s="0" t="s">
+      <c r="F67" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M67" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="N67" s="0" t="s">
+      <c r="M67" s="14" t="s">
         <v>78</v>
       </c>
+      <c r="N67" s="1" t="s">
+        <v>76</v>
+      </c>
       <c r="O67" s="15" t="n">
-        <v>18.194124</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O68" s="15"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F69" s="0" t="s">
+      <c r="F69" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M69" s="16" t="s">
+      <c r="M69" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N69" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O69" s="15" t="n">
+        <v>2.424</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F70" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M70" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N70" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O70" s="15" t="n">
+        <v>2.128</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F71" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M71" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N71" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O71" s="15" t="n">
+        <v>2.246666667</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F72" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M72" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N72" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O72" s="15" t="n">
+        <v>1.936</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F73" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M73" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N73" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O73" s="15" t="n">
+        <v>8.208</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F74" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M74" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N74" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O74" s="15" t="n">
+        <v>6.152</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F75" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M75" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="N75" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O75" s="15" t="n">
+        <v>2.64</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O76" s="15"/>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F77" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M77" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N69" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O69" s="17" t="n">
-        <v>7.55</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F70" s="0" t="s">
+      <c r="N77" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O77" s="15" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F78" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M70" s="16" t="s">
+      <c r="M78" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N70" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O70" s="17" t="n">
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F71" s="0" t="s">
+      <c r="N78" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O78" s="15" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F79" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M71" s="16" t="s">
+      <c r="M79" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N71" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O71" s="17" t="n">
-        <v>6.566666667</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F72" s="0" t="s">
+      <c r="N79" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O79" s="15" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F80" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M72" s="16" t="s">
+      <c r="M80" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N72" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O72" s="17" t="n">
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F73" s="0" t="s">
+      <c r="N80" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O80" s="15" t="n">
+        <v>0.345</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F81" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M73" s="16" t="s">
+      <c r="M81" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N73" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O73" s="17" t="n">
-        <v>7.15</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F74" s="0" t="s">
+      <c r="N81" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O81" s="15" t="n">
+        <v>0.715</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F82" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M74" s="16" t="s">
+      <c r="M82" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N74" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O74" s="17" t="n">
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F75" s="0" t="s">
+      <c r="N82" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O82" s="15" t="n">
+        <v>1.245</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F83" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M75" s="16" t="s">
+      <c r="M83" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="N75" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O75" s="17" t="n">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O76" s="17"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F77" s="0" t="s">
+      <c r="N83" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O83" s="15" t="n">
+        <v>1.195</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O84" s="15"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F85" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M77" s="16" t="s">
+      <c r="M85" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N77" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O77" s="17" t="n">
-        <v>2.424</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F78" s="0" t="s">
+      <c r="N85" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O85" s="15" t="n">
+        <v>2.425</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F86" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M78" s="16" t="s">
+      <c r="M86" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N78" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O78" s="17" t="n">
-        <v>2.128</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F79" s="0" t="s">
+      <c r="N86" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O86" s="15" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F87" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M79" s="16" t="s">
+      <c r="M87" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N79" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O79" s="17" t="n">
-        <v>2.246666667</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F80" s="0" t="s">
+      <c r="N87" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O87" s="15" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F88" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M80" s="16" t="s">
+      <c r="M88" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N80" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O80" s="17" t="n">
-        <v>1.936</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F81" s="0" t="s">
+      <c r="N88" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O88" s="15" t="n">
+        <v>0.525</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F89" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M81" s="16" t="s">
+      <c r="M89" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N81" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O81" s="17" t="n">
-        <v>8.208</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F82" s="0" t="s">
+      <c r="N89" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O89" s="15" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F90" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M82" s="16" t="s">
+      <c r="M90" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N82" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O82" s="17" t="n">
-        <v>6.152</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F83" s="0" t="s">
+      <c r="N90" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O90" s="15" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F91" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M83" s="16" t="s">
+      <c r="M91" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="N83" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O83" s="17" t="n">
-        <v>2.64</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O84" s="17"/>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F85" s="0" t="s">
+      <c r="N91" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O91" s="15" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O92" s="13"/>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="O93" s="13"/>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F94" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M85" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N85" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O85" s="17" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F86" s="0" t="s">
+      <c r="M94" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N94" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O94" s="13" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="P94" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q94" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F95" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M86" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N86" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O86" s="17" t="n">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F87" s="0" t="s">
+      <c r="M95" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N95" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O95" s="13" t="n">
+        <v>10.1</v>
+      </c>
+      <c r="Q95" s="10"/>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F96" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M87" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N87" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O87" s="17" t="n">
-        <v>0.27</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F88" s="0" t="s">
+      <c r="M96" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N96" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O96" s="13" t="n">
+        <v>9.941666667</v>
+      </c>
+      <c r="Q96" s="10"/>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F97" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M88" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N88" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O88" s="17" t="n">
-        <v>0.345</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F89" s="0" t="s">
+      <c r="M97" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N97" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O97" s="13" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="Q97" s="10"/>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F98" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M89" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N89" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O89" s="17" t="n">
-        <v>0.715</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F90" s="0" t="s">
+      <c r="M98" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N98" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O98" s="13" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="Q98" s="10"/>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F99" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M90" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N90" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O90" s="17" t="n">
-        <v>1.245</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F91" s="0" t="s">
+      <c r="M99" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N99" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O99" s="13" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q99" s="10"/>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F100" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M91" s="16" t="s">
-        <v>82</v>
-      </c>
-      <c r="N91" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O91" s="17" t="n">
-        <v>1.195</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O92" s="17"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F93" s="0" t="s">
+      <c r="M100" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="N100" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O100" s="13" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q100" s="10"/>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O101" s="16"/>
+      <c r="Q101" s="10"/>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F102" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M93" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N93" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O93" s="17" t="n">
-        <v>2.425</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F94" s="0" t="s">
+      <c r="M102" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N102" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O102" s="13" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="P102" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q102" s="11"/>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F103" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M94" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N94" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O94" s="17" t="n">
-        <v>2.34</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F95" s="0" t="s">
+      <c r="M103" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N103" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O103" s="13" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="Q103" s="11"/>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F104" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M95" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N95" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O95" s="17" t="n">
-        <v>2.34</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F96" s="0" t="s">
+      <c r="M104" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N104" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O104" s="13" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="Q104" s="11"/>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F105" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M96" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N96" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O96" s="17" t="n">
-        <v>0.525</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F97" s="0" t="s">
+      <c r="M105" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N105" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O105" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q105" s="11"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F106" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M97" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N97" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O97" s="17" t="n">
-        <v>2.35</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F98" s="0" t="s">
+      <c r="M106" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N106" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O106" s="13" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="Q106" s="11"/>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F107" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M98" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N98" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O98" s="17" t="n">
-        <v>1.55</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F99" s="0" t="s">
+      <c r="M107" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N107" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O107" s="13" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="Q107" s="11"/>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F108" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M99" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="N99" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O99" s="17" t="n">
-        <v>1.35</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O100" s="15"/>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="O101" s="15"/>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F102" s="0" t="s">
+      <c r="M108" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="N108" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O108" s="13" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="Q108" s="11"/>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O109" s="16"/>
+      <c r="Q109" s="11"/>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F110" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M102" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N102" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O102" s="15" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="P102" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q102" s="10" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F103" s="0" t="s">
+      <c r="M110" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N110" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O110" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="P110" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q110" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F111" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="M103" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N103" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O103" s="15" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="Q103" s="10"/>
-    </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F104" s="0" t="s">
+      <c r="M111" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N111" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O111" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q111" s="10"/>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F112" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="M104" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N104" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O104" s="15" t="n">
-        <v>9.941666667</v>
-      </c>
-      <c r="Q104" s="10"/>
-    </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F105" s="0" t="s">
+      <c r="M112" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N112" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O112" s="13" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q112" s="11"/>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F113" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="M105" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N105" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O105" s="15" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="Q105" s="10"/>
-    </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F106" s="0" t="s">
+      <c r="M113" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N113" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O113" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F114" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="M106" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N106" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O106" s="15" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="Q106" s="10"/>
-    </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F107" s="0" t="s">
+      <c r="M114" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N114" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O114" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q114" s="10"/>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F115" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="M107" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N107" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O107" s="15" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="Q107" s="10"/>
-    </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F108" s="0" t="s">
+      <c r="M115" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N115" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O115" s="13" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q115" s="11"/>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="F116" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M108" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="N108" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O108" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q108" s="10"/>
-    </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O109" s="18"/>
-      <c r="Q109" s="10"/>
-    </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F110" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="M110" s="0" t="s">
+      <c r="M116" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="N110" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O110" s="15" t="n">
-        <v>13.35</v>
-      </c>
-      <c r="P110" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q110" s="11"/>
-    </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F111" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="M111" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N111" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O111" s="15" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="Q111" s="11"/>
-    </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F112" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="M112" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N112" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O112" s="15" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="Q112" s="11"/>
-    </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F113" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="M113" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N113" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O113" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q113" s="11"/>
-    </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F114" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="M114" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N114" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O114" s="15" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="Q114" s="11"/>
-    </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F115" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="M115" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N115" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O115" s="15" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="Q115" s="11"/>
-    </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F116" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="M116" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="N116" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O116" s="15" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="Q116" s="11"/>
+      <c r="N116" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="O116" s="13" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O117" s="18"/>
-      <c r="Q117" s="11"/>
+      <c r="O117" s="10"/>
+      <c r="Q117" s="10"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F118" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="M118" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N118" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O118" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="P118" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q118" s="10" t="s">
-        <v>92</v>
-      </c>
+      <c r="O118" s="10"/>
+      <c r="Q118" s="11"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F119" s="0" t="s">
-        <v>30</v>
-      </c>
-      <c r="M119" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N119" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O119" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q119" s="10"/>
+      <c r="L119" s="8"/>
+      <c r="M119" s="8"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F120" s="0" t="s">
-        <v>31</v>
-      </c>
-      <c r="M120" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N120" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O120" s="15" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q120" s="11"/>
-    </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F121" s="0" t="s">
-        <v>32</v>
-      </c>
-      <c r="M121" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N121" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O121" s="15" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F122" s="0" t="s">
-        <v>34</v>
-      </c>
-      <c r="M122" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N122" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O122" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q122" s="10"/>
-    </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F123" s="0" t="s">
-        <v>35</v>
-      </c>
-      <c r="M123" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N123" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O123" s="15" t="n">
-        <v>46</v>
-      </c>
-      <c r="Q123" s="11"/>
-    </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="0" t="s">
-        <v>48</v>
-      </c>
-      <c r="F124" s="0" t="s">
-        <v>36</v>
-      </c>
-      <c r="M124" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="N124" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="O124" s="15" t="n">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O125" s="10"/>
-      <c r="Q125" s="10"/>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O126" s="10"/>
-      <c r="Q126" s="11"/>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L127" s="8"/>
-      <c r="M127" s="8"/>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O128" s="10"/>
-      <c r="Q128" s="10"/>
-    </row>
+      <c r="O120" s="10"/>
+      <c r="Q120" s="10"/>
+    </row>
+    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Update mini data for new feed structure
</commit_message>
<xml_diff>
--- a/mini/data/default/FeedMgmt.xlsx
+++ b/mini/data/default/FeedMgmt.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="341" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="98">
   <si>
     <t xml:space="preserve">Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
   </si>
@@ -182,6 +182,12 @@
     <t xml:space="preserve">%</t>
   </si>
   <si>
+    <t xml:space="preserve">conventional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">organic</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -224,6 +230,15 @@
     <t xml:space="preserve">share_imported</t>
   </si>
   <si>
+    <t xml:space="preserve">Max total amounts of crop and by-products that are imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_total_imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg product</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -353,7 +368,7 @@
     <t xml:space="preserve">Cattle</t>
   </si>
   <si>
-    <t xml:space="preserve">E</t>
+    <t xml:space="preserve">ME</t>
   </si>
   <si>
     <t xml:space="preserve">MJ ME/kg DM</t>
@@ -375,6 +390,12 @@
   </si>
   <si>
     <t xml:space="preserve">Total fat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g AAT/kg DM</t>
   </si>
 </sst>
 </file>
@@ -387,7 +408,7 @@
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -462,6 +483,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -511,7 +539,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -561,6 +589,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1173,6 +1205,9 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C20" s="1" t="s">
+        <v>43</v>
+      </c>
       <c r="I20" s="1" t="s">
         <v>31</v>
       </c>
@@ -1187,37 +1222,39 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O21" s="11"/>
-      <c r="Q21" s="11"/>
-    </row>
-    <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>43</v>
-      </c>
+      <c r="C21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O21" s="11" t="n">
+        <v>50</v>
+      </c>
+      <c r="P21" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O22" s="11"/>
       <c r="Q22" s="11"/>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I23" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="O23" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="P23" s="1" t="s">
-        <v>42</v>
-      </c>
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="O23" s="11"/>
       <c r="Q23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I24" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="N24" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="O24" s="11" t="n">
         <v>5</v>
@@ -1228,1371 +1265,1585 @@
       <c r="Q24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O25" s="11"/>
+      <c r="I25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="O25" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="P25" s="1" t="s">
+        <v>42</v>
+      </c>
       <c r="Q25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4"/>
-      <c r="K26" s="4"/>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-      <c r="R26" s="4"/>
+      <c r="O26" s="11"/>
+      <c r="Q26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N27" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="O27" s="6" t="n">
+      <c r="A27" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
+      <c r="K27" s="4"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="4"/>
+      <c r="O27" s="4"/>
+      <c r="P27" s="4"/>
+      <c r="Q27" s="4"/>
+      <c r="R27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N28" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="O28" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="P27" s="6" t="s">
+      <c r="P28" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="Q27" s="6" t="s">
+      <c r="Q28" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="4"/>
-      <c r="N28" s="4"/>
-      <c r="O28" s="4"/>
-      <c r="P28" s="4"/>
-      <c r="Q28" s="4"/>
-      <c r="R28" s="4"/>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
+      <c r="K29" s="4"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="4"/>
+      <c r="O29" s="4"/>
+      <c r="P29" s="4"/>
+      <c r="Q29" s="4"/>
+      <c r="R29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I30" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N30" s="1" t="s">
+      <c r="N30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O30" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="P30" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q30" s="10"/>
+      <c r="O30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q30" s="6" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E31" s="1" t="s">
+      <c r="C31" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N31" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="O31" s="13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="P31" s="13"/>
+      <c r="Q31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C32" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="N32" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="O32" s="13" t="n">
+        <v>200000</v>
+      </c>
+      <c r="P32" s="13"/>
+      <c r="Q32" s="6"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N33" s="6"/>
+      <c r="O33" s="6"/>
+      <c r="P33" s="6"/>
+      <c r="Q33" s="6"/>
+    </row>
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H31" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="N31" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="O31" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="P31" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q31" s="10"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O32" s="11"/>
-      <c r="Q32" s="11"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="4"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N34" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="O34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P34" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q34" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N35" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="O35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P35" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q35" s="6" t="s">
-        <v>26</v>
-      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
+      <c r="I34" s="4"/>
+      <c r="J34" s="4"/>
+      <c r="K34" s="4"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="4"/>
+      <c r="O34" s="4"/>
+      <c r="P34" s="4"/>
+      <c r="Q34" s="4"/>
+      <c r="R34" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N36" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O36" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="P36" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q36" s="10"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="N36" s="10" t="s">
+      <c r="E37" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="H37" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="O36" s="10" t="n">
+      <c r="I37" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="N37" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O37" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="P37" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q37" s="10"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O38" s="11"/>
+      <c r="Q38" s="11"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
+      <c r="K39" s="4"/>
+      <c r="L39" s="4"/>
+      <c r="M39" s="4"/>
+      <c r="N39" s="4"/>
+      <c r="O39" s="4"/>
+      <c r="P39" s="4"/>
+      <c r="Q39" s="4"/>
+      <c r="R39" s="4"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N40" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q40" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N41" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q41" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N42" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="O42" s="10" t="n">
         <f aca="false">(0.8*20+0.2*2)</f>
         <v>16.4</v>
       </c>
-      <c r="P36" s="10" t="s">
+      <c r="P42" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Q36" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="R36" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="N37" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="O37" s="10" t="n">
+      <c r="Q42" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="R42" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N43" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="O43" s="10" t="n">
         <f aca="false">(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
-      <c r="P37" s="10" t="s">
+      <c r="P43" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Q37" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="R37" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N38" s="10"/>
-      <c r="O38" s="10"/>
-      <c r="P38" s="10"/>
-      <c r="Q38" s="10"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="G39" s="1" t="s">
+      <c r="Q43" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="R43" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="10"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="N39" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="O39" s="10" t="n">
+      <c r="E45" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N45" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="O45" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="P39" s="10" t="s">
+      <c r="P45" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Q39" s="10" t="s">
+      <c r="Q45" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="R45" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="N46" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="R39" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E40" s="1" t="s">
+      <c r="O46" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="P46" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q46" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="R46" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G47" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="G40" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="N40" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="O40" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="P40" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q40" s="10" t="s">
+      <c r="N47" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="R40" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="N41" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="O41" s="10" t="n">
+      <c r="O47" s="10" t="n">
         <f aca="false">0.9*5+0.1*15</f>
         <v>6</v>
       </c>
-      <c r="P41" s="10" t="s">
+      <c r="P47" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Q41" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="R41" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N42" s="10"/>
-      <c r="O42" s="10"/>
-      <c r="P42" s="10"/>
-      <c r="Q42" s="10"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11"/>
-      <c r="G43" s="1" t="s">
+      <c r="Q47" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="R47" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="N43" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="O43" s="10"/>
-      <c r="Q43" s="11" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11"/>
-      <c r="G44" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="N44" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="O44" s="10" t="n">
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N48" s="10"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="10"/>
+      <c r="Q48" s="10"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="11"/>
+      <c r="G49" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="N49" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="O49" s="10"/>
+      <c r="Q49" s="11" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="11"/>
+      <c r="G50" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="N50" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="O50" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="P44" s="10" t="s">
+      <c r="P50" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="Q44" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="R44" s="1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="11"/>
-      <c r="N45" s="10"/>
-      <c r="O45" s="10"/>
-      <c r="P45" s="10"/>
-      <c r="Q45" s="11"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="3"/>
-      <c r="D46" s="3"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-      <c r="J46" s="4"/>
-      <c r="K46" s="4"/>
-      <c r="L46" s="4"/>
-      <c r="M46" s="4"/>
-      <c r="N46" s="4"/>
-      <c r="O46" s="4"/>
-      <c r="P46" s="4"/>
-      <c r="Q46" s="4"/>
-      <c r="R46" s="4"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O47" s="10"/>
-      <c r="Q47" s="10" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O48" s="10"/>
-      <c r="Q48" s="11"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N49" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="O49" s="10" t="n">
+      <c r="Q50" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="R50" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="11"/>
+      <c r="N51" s="10"/>
+      <c r="O51" s="10"/>
+      <c r="P51" s="10"/>
+      <c r="Q51" s="11"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="4"/>
+      <c r="F52" s="4"/>
+      <c r="G52" s="4"/>
+      <c r="H52" s="4"/>
+      <c r="I52" s="4"/>
+      <c r="J52" s="4"/>
+      <c r="K52" s="4"/>
+      <c r="L52" s="4"/>
+      <c r="M52" s="4"/>
+      <c r="N52" s="4"/>
+      <c r="O52" s="4"/>
+      <c r="P52" s="4"/>
+      <c r="Q52" s="4"/>
+      <c r="R52" s="4"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="O53" s="10"/>
+      <c r="Q53" s="10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O54" s="10"/>
+      <c r="Q54" s="11"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="N55" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="O55" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="P49" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q49" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="R49" s="10"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O50" s="11"/>
-      <c r="Q50" s="11"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="3"/>
-      <c r="D51" s="3"/>
-      <c r="E51" s="4"/>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
-      <c r="H51" s="4"/>
-      <c r="I51" s="4"/>
-      <c r="J51" s="4"/>
-      <c r="K51" s="4"/>
-      <c r="L51" s="4"/>
-      <c r="M51" s="4"/>
-      <c r="N51" s="4"/>
-      <c r="O51" s="4"/>
-      <c r="P51" s="4"/>
-      <c r="Q51" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="R51" s="4"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F53" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M53" s="1" t="s">
+      <c r="P55" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="N53" s="1" t="s">
+      <c r="Q55" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="O53" s="13" t="n">
-        <v>17.3169484</v>
-      </c>
-      <c r="P53" s="1" t="s">
+      <c r="R55" s="10"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O56" s="11"/>
+      <c r="Q56" s="11"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F54" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M54" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N54" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O54" s="13" t="n">
-        <v>17.150216</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F55" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M55" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N55" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O55" s="13" t="n">
-        <v>17.41143707</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F56" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M56" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N56" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O56" s="13" t="n">
-        <v>18.2100232</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F57" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N57" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O57" s="13" t="n">
-        <v>19.589488</v>
-      </c>
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="4"/>
+      <c r="F57" s="4"/>
+      <c r="G57" s="4"/>
+      <c r="H57" s="4"/>
+      <c r="I57" s="4"/>
+      <c r="J57" s="4"/>
+      <c r="K57" s="4"/>
+      <c r="L57" s="4"/>
+      <c r="M57" s="4"/>
+      <c r="N57" s="4"/>
+      <c r="O57" s="4"/>
+      <c r="P57" s="4"/>
+      <c r="Q57" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="R57" s="4"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F58" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M58" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="N58" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O58" s="13" t="n">
-        <v>19.4920008</v>
+      <c r="A58" s="8" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F59" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M59" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O59" s="13" t="n">
-        <v>18.194124</v>
+        <v>81</v>
+      </c>
+      <c r="O59" s="14" t="n">
+        <v>17.3169484</v>
+      </c>
+      <c r="P59" s="1" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O60" s="13"/>
+      <c r="F60" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M60" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="N60" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O60" s="14" t="n">
+        <v>17.150216</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F61" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M61" s="14" t="s">
-        <v>78</v>
+        <v>31</v>
+      </c>
+      <c r="M61" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="N61" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O61" s="15" t="n">
-        <v>7.55</v>
+        <v>81</v>
+      </c>
+      <c r="O61" s="14" t="n">
+        <v>17.41143707</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F62" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M62" s="14" t="s">
-        <v>78</v>
+        <v>32</v>
+      </c>
+      <c r="M62" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="N62" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O62" s="15" t="n">
-        <v>7.8</v>
+        <v>81</v>
+      </c>
+      <c r="O62" s="14" t="n">
+        <v>18.2100232</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F63" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M63" s="14" t="s">
-        <v>78</v>
+        <v>34</v>
+      </c>
+      <c r="M63" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="N63" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O63" s="15" t="n">
-        <v>6.566666667</v>
+        <v>81</v>
+      </c>
+      <c r="O63" s="14" t="n">
+        <v>19.589488</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F64" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M64" s="14" t="s">
-        <v>78</v>
+        <v>35</v>
+      </c>
+      <c r="M64" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="N64" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O64" s="15" t="n">
-        <v>1.8</v>
+        <v>81</v>
+      </c>
+      <c r="O64" s="14" t="n">
+        <v>19.4920008</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F65" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M65" s="14" t="s">
-        <v>78</v>
+        <v>36</v>
+      </c>
+      <c r="M65" s="1" t="s">
+        <v>80</v>
       </c>
       <c r="N65" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O65" s="15" t="n">
-        <v>7.15</v>
+        <v>81</v>
+      </c>
+      <c r="O65" s="14" t="n">
+        <v>18.194124</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F66" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M66" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="N66" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O66" s="15" t="n">
-        <v>7.7</v>
-      </c>
+      <c r="O66" s="14"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F67" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="M67" s="14" t="s">
-        <v>78</v>
+        <v>28</v>
+      </c>
+      <c r="M67" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N67" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O67" s="15" t="n">
-        <v>5.9</v>
+        <v>81</v>
+      </c>
+      <c r="O67" s="16" t="n">
+        <v>7.55</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O68" s="15"/>
+      <c r="F68" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M68" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="N68" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O68" s="16" t="n">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F69" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M69" s="14" t="s">
-        <v>79</v>
+        <v>31</v>
+      </c>
+      <c r="M69" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N69" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O69" s="15" t="n">
-        <v>2.424</v>
+        <v>81</v>
+      </c>
+      <c r="O69" s="16" t="n">
+        <v>6.566666667</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F70" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M70" s="14" t="s">
-        <v>79</v>
+        <v>32</v>
+      </c>
+      <c r="M70" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N70" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O70" s="15" t="n">
-        <v>2.128</v>
+        <v>81</v>
+      </c>
+      <c r="O70" s="16" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F71" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M71" s="14" t="s">
-        <v>79</v>
+        <v>34</v>
+      </c>
+      <c r="M71" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N71" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O71" s="15" t="n">
-        <v>2.246666667</v>
+        <v>81</v>
+      </c>
+      <c r="O71" s="16" t="n">
+        <v>7.15</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F72" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M72" s="14" t="s">
-        <v>79</v>
+        <v>35</v>
+      </c>
+      <c r="M72" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N72" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O72" s="15" t="n">
-        <v>1.936</v>
+        <v>81</v>
+      </c>
+      <c r="O72" s="16" t="n">
+        <v>7.7</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F73" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M73" s="14" t="s">
-        <v>79</v>
+        <v>36</v>
+      </c>
+      <c r="M73" s="15" t="s">
+        <v>83</v>
       </c>
       <c r="N73" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O73" s="15" t="n">
-        <v>8.208</v>
+        <v>81</v>
+      </c>
+      <c r="O73" s="16" t="n">
+        <v>5.9</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F74" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M74" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="N74" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O74" s="15" t="n">
-        <v>6.152</v>
-      </c>
+      <c r="O74" s="16"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F75" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="M75" s="14" t="s">
-        <v>79</v>
+        <v>28</v>
+      </c>
+      <c r="M75" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N75" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O75" s="15" t="n">
-        <v>2.64</v>
+        <v>81</v>
+      </c>
+      <c r="O75" s="16" t="n">
+        <v>2.424</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O76" s="15"/>
+      <c r="F76" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M76" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="N76" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O76" s="16" t="n">
+        <v>2.128</v>
+      </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F77" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M77" s="14" t="s">
-        <v>80</v>
+        <v>31</v>
+      </c>
+      <c r="M77" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N77" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O77" s="15" t="n">
-        <v>0.28</v>
+        <v>81</v>
+      </c>
+      <c r="O77" s="16" t="n">
+        <v>2.246666667</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F78" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M78" s="14" t="s">
-        <v>80</v>
+        <v>32</v>
+      </c>
+      <c r="M78" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N78" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O78" s="15" t="n">
-        <v>0.27</v>
+        <v>81</v>
+      </c>
+      <c r="O78" s="16" t="n">
+        <v>1.936</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F79" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M79" s="14" t="s">
-        <v>80</v>
+        <v>34</v>
+      </c>
+      <c r="M79" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N79" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O79" s="15" t="n">
-        <v>0.27</v>
+        <v>81</v>
+      </c>
+      <c r="O79" s="16" t="n">
+        <v>8.208</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F80" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M80" s="14" t="s">
-        <v>80</v>
+        <v>35</v>
+      </c>
+      <c r="M80" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N80" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O80" s="15" t="n">
-        <v>0.345</v>
+        <v>81</v>
+      </c>
+      <c r="O80" s="16" t="n">
+        <v>6.152</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F81" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M81" s="14" t="s">
-        <v>80</v>
+        <v>36</v>
+      </c>
+      <c r="M81" s="15" t="s">
+        <v>84</v>
       </c>
       <c r="N81" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O81" s="15" t="n">
-        <v>0.715</v>
+        <v>81</v>
+      </c>
+      <c r="O81" s="16" t="n">
+        <v>2.64</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F82" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M82" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="N82" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O82" s="15" t="n">
-        <v>1.245</v>
-      </c>
+      <c r="O82" s="16"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F83" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="M83" s="14" t="s">
-        <v>80</v>
+        <v>28</v>
+      </c>
+      <c r="M83" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N83" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O83" s="15" t="n">
-        <v>1.195</v>
+        <v>81</v>
+      </c>
+      <c r="O83" s="16" t="n">
+        <v>0.28</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O84" s="15"/>
+      <c r="F84" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M84" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="N84" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O84" s="16" t="n">
+        <v>0.27</v>
+      </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F85" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M85" s="14" t="s">
-        <v>81</v>
+        <v>31</v>
+      </c>
+      <c r="M85" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N85" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O85" s="15" t="n">
-        <v>2.425</v>
+        <v>81</v>
+      </c>
+      <c r="O85" s="16" t="n">
+        <v>0.27</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F86" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M86" s="14" t="s">
-        <v>81</v>
+        <v>32</v>
+      </c>
+      <c r="M86" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N86" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O86" s="15" t="n">
-        <v>2.34</v>
+        <v>81</v>
+      </c>
+      <c r="O86" s="16" t="n">
+        <v>0.345</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F87" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M87" s="14" t="s">
-        <v>81</v>
+        <v>34</v>
+      </c>
+      <c r="M87" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N87" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O87" s="15" t="n">
-        <v>2.34</v>
+        <v>81</v>
+      </c>
+      <c r="O87" s="16" t="n">
+        <v>0.715</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F88" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M88" s="14" t="s">
-        <v>81</v>
+        <v>35</v>
+      </c>
+      <c r="M88" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N88" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O88" s="15" t="n">
-        <v>0.525</v>
+        <v>81</v>
+      </c>
+      <c r="O88" s="16" t="n">
+        <v>1.245</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F89" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M89" s="14" t="s">
-        <v>81</v>
+        <v>36</v>
+      </c>
+      <c r="M89" s="15" t="s">
+        <v>85</v>
       </c>
       <c r="N89" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O89" s="15" t="n">
-        <v>2.35</v>
+        <v>81</v>
+      </c>
+      <c r="O89" s="16" t="n">
+        <v>1.195</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F90" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M90" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="N90" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O90" s="15" t="n">
-        <v>1.55</v>
-      </c>
+      <c r="O90" s="16"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F91" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M91" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N91" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O91" s="16" t="n">
+        <v>2.425</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F92" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M92" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N92" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O92" s="16" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F93" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M93" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N93" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O93" s="16" t="n">
+        <v>2.34</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F94" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M94" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N94" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O94" s="16" t="n">
+        <v>0.525</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F95" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M95" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N95" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O95" s="16" t="n">
+        <v>2.35</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F96" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M96" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N96" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O96" s="16" t="n">
+        <v>1.55</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F97" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M91" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="N91" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O91" s="15" t="n">
+      <c r="M97" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="N97" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O97" s="16" t="n">
         <v>1.35</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O92" s="13"/>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="O93" s="13"/>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F94" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M94" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N94" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O94" s="13" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="P94" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="Q94" s="10" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F95" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="M95" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N95" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O95" s="13" t="n">
-        <v>10.1</v>
-      </c>
-      <c r="Q95" s="10"/>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F96" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="M96" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N96" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O96" s="13" t="n">
-        <v>9.941666667</v>
-      </c>
-      <c r="Q96" s="10"/>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M97" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N97" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O97" s="13" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="Q97" s="10"/>
-    </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F98" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M98" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N98" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O98" s="13" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="Q98" s="10"/>
+      <c r="O98" s="14"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F99" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M99" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="N99" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O99" s="13" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="Q99" s="10"/>
+      <c r="A99" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="O99" s="14"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M100" s="1" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="N100" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O100" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q100" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="O100" s="14" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="P100" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q100" s="10" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O101" s="16"/>
+      <c r="A101" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M101" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="N101" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O101" s="14" t="n">
+        <v>10.1</v>
+      </c>
       <c r="Q101" s="10"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="M102" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N102" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O102" s="13" t="n">
-        <v>13.35</v>
-      </c>
-      <c r="P102" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="Q102" s="11"/>
+        <v>81</v>
+      </c>
+      <c r="O102" s="14" t="n">
+        <v>9.941666667</v>
+      </c>
+      <c r="Q102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M103" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N103" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O103" s="13" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="Q103" s="11"/>
+        <v>81</v>
+      </c>
+      <c r="O103" s="14" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="Q103" s="10"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="M104" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N104" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O104" s="13" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="Q104" s="11"/>
+        <v>81</v>
+      </c>
+      <c r="O104" s="14" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="Q104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="M105" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N105" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O105" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q105" s="11"/>
+        <v>81</v>
+      </c>
+      <c r="O105" s="14" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="Q105" s="10"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M106" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N106" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O106" s="13" t="n">
-        <v>17.8</v>
-      </c>
-      <c r="Q106" s="11"/>
+        <v>81</v>
+      </c>
+      <c r="O106" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F107" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M107" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="N107" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O107" s="13" t="n">
-        <v>14.6</v>
-      </c>
-      <c r="Q107" s="11"/>
+      <c r="O107" s="17"/>
+      <c r="Q107" s="10"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="M108" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="N108" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O108" s="13" t="n">
-        <v>12.7</v>
+        <v>81</v>
+      </c>
+      <c r="O108" s="14" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="P108" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="Q108" s="11"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O109" s="16"/>
+      <c r="A109" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M109" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="N109" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O109" s="14" t="n">
+        <v>11.9</v>
+      </c>
       <c r="Q109" s="11"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="M110" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N110" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O110" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="P110" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="Q110" s="10" t="s">
-        <v>90</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="O110" s="14" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="Q110" s="11"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M111" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N111" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O111" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="Q111" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="O111" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q111" s="11"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="M112" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N112" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O112" s="13" t="n">
-        <v>20</v>
+        <v>81</v>
+      </c>
+      <c r="O112" s="14" t="n">
+        <v>17.8</v>
       </c>
       <c r="Q112" s="11"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="M113" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N113" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O113" s="13" t="n">
-        <v>25</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="O113" s="14" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="Q113" s="11"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="M114" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="N114" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O114" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q114" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="O114" s="14" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="Q114" s="11"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="M115" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N115" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O115" s="13" t="n">
-        <v>46</v>
-      </c>
+      <c r="O115" s="17"/>
       <c r="Q115" s="11"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="F116" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M116" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N116" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O116" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="P116" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q116" s="10" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M117" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N117" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O117" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q117" s="10"/>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M118" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N118" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O118" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q118" s="11"/>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M119" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N119" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O119" s="14" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M120" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N120" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O120" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q120" s="10"/>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M121" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N121" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O121" s="14" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q121" s="11"/>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F122" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="M116" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="N116" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="O116" s="13" t="n">
+      <c r="M122" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="N122" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O122" s="14" t="n">
         <v>45</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O117" s="10"/>
-      <c r="Q117" s="10"/>
-    </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O118" s="10"/>
-      <c r="Q118" s="11"/>
-    </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L119" s="8"/>
-      <c r="M119" s="8"/>
-    </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O120" s="10"/>
-      <c r="Q120" s="10"/>
-    </row>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O123" s="10"/>
+      <c r="Q123" s="10"/>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M124" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N124" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O124" s="14" t="n">
+        <v>72</v>
+      </c>
+      <c r="P124" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q124" s="11"/>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L125" s="8"/>
+      <c r="M125" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N125" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O125" s="14" t="n">
+        <v>69</v>
+      </c>
+      <c r="P125" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M126" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N126" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O126" s="14" t="n">
+        <v>74.3333333333333</v>
+      </c>
+      <c r="P126" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q126" s="10"/>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M127" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N127" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O127" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="P127" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M128" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N128" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O128" s="14" t="n">
+        <v>182</v>
+      </c>
+      <c r="P128" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M129" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N129" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O129" s="14" t="n">
+        <v>221</v>
+      </c>
+      <c r="P129" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M130" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="N130" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O130" s="14" t="n">
+        <v>73</v>
+      </c>
+      <c r="P130" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>

</xml_diff>

<commit_message>
Added PBV values for feeds
</commit_message>
<xml_diff>
--- a/mini/data/default/FeedMgmt.xlsx
+++ b/mini/data/default/FeedMgmt.xlsx
@@ -1,17 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\mini\data\default\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="references" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="default" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="references" sheetId="1" r:id="rId1"/>
+    <sheet name="default" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -21,126 +25,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="391" uniqueCount="98">
-  <si>
-    <t xml:space="preserve">Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cederberg, C. &amp; Henriksson, M. (2020). Gräsmarkernas användning i jordbruket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hessle, A. &amp; Danielsson, R. (2023) Number of cattle required to obtain good ecological status in Swedish grasslands and livestock’s methane emissions. Swedish University of Agricultural Sciences. Department of Animal Environment and Health. Section of Production systems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_species</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_breed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_prod_system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_sub_system</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_animal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_feed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_feed_group:feed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_crop_group</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_crop_prod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_by_prod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_crop_resid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_region</t>
-  </si>
-  <si>
-    <t xml:space="preserve">f_feed_par</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parameter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conversion factors: Feeds --&gt; crop products, by-products or crop residues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg product/kg DM feed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">need to align with DM in products and by-products</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feed_to_prod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fallback</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crop products</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ley silage, 1st cut</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fodder</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ley silage, regrowth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">grazing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wheat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">By-products</t>
-  </si>
-  <si>
-    <t xml:space="preserve">soybean meal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rapeseed meal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wheat bran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">milling by-products from wheat, barley or rye</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crop residues</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameters to constrain regional feed supply</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="100">
+  <si>
+    <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
+  </si>
+  <si>
+    <t>Cederberg, C. &amp; Henriksson, M. (2020). Gräsmarkernas användning i jordbruket</t>
+  </si>
+  <si>
+    <t>Hessle, A. &amp; Danielsson, R. (2023) Number of cattle required to obtain good ecological status in Swedish grasslands and livestock’s methane emissions. Swedish University of Agricultural Sciences. Department of Animal Environment and Health. Section of Production systems</t>
+  </si>
+  <si>
+    <t>Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
+  </si>
+  <si>
+    <t>f_species</t>
+  </si>
+  <si>
+    <t>f_breed</t>
+  </si>
+  <si>
+    <t>f_prod_system</t>
+  </si>
+  <si>
+    <t>f_sub_system</t>
+  </si>
+  <si>
+    <t>f_animal</t>
+  </si>
+  <si>
+    <t>f_feed</t>
+  </si>
+  <si>
+    <t>f_feed_group:feed</t>
+  </si>
+  <si>
+    <t>f_crop_group</t>
+  </si>
+  <si>
+    <t>f_crop_prod</t>
+  </si>
+  <si>
+    <t>f_by_prod</t>
+  </si>
+  <si>
+    <t>f_crop_resid</t>
+  </si>
+  <si>
+    <t>f_region</t>
+  </si>
+  <si>
+    <t>f_feed_par</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>source</t>
+  </si>
+  <si>
+    <t>Conversion factors: Feeds --&gt; crop products, by-products or crop residues</t>
+  </si>
+  <si>
+    <t>kg product/kg DM feed</t>
+  </si>
+  <si>
+    <t>need to align with DM in products and by-products</t>
+  </si>
+  <si>
+    <t>feed_to_prod</t>
+  </si>
+  <si>
+    <t>fallback</t>
+  </si>
+  <si>
+    <t>Crop products</t>
+  </si>
+  <si>
+    <t>ley silage, 1st cut</t>
+  </si>
+  <si>
+    <t>fodder</t>
+  </si>
+  <si>
+    <t>ley silage, regrowth</t>
+  </si>
+  <si>
+    <t>grazing</t>
+  </si>
+  <si>
+    <t>wheat</t>
+  </si>
+  <si>
+    <t>By-products</t>
+  </si>
+  <si>
+    <t>soybean meal</t>
+  </si>
+  <si>
+    <t>rapeseed meal</t>
+  </si>
+  <si>
+    <t>wheat bran</t>
+  </si>
+  <si>
+    <t>milling by-products from wheat, barley or rye</t>
+  </si>
+  <si>
+    <t>Crop residues</t>
+  </si>
+  <si>
+    <t>Parameters to constrain regional feed supply</t>
   </si>
   <si>
     <r>
@@ -151,11 +155,11 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">The parameter</t>
+      <t>The parameter</t>
     </r>
     <r>
       <rPr>
-        <b val="true"/>
+        <b/>
         <sz val="11"/>
         <color theme="4"/>
         <rFont val="Calibri"/>
@@ -176,16 +180,16 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">share_regional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">conventional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">organic</t>
+    <t>share_regional</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>conventional</t>
+  </si>
+  <si>
+    <t>organic</t>
   </si>
   <si>
     <r>
@@ -200,14 +204,14 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
+        <b/>
         <sz val="11"/>
         <color theme="4"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">max_overproduction</t>
+      <t>max_overproduction</t>
     </r>
     <r>
       <rPr>
@@ -221,35 +225,35 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">max_overproduction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share of crop and by-products that are imported</t>
-  </si>
-  <si>
-    <t xml:space="preserve">share_imported</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Max total amounts of crop and by-products that are imported</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_total_imported</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg product</t>
+    <t>max_overproduction</t>
+  </si>
+  <si>
+    <t>Share of crop and by-products that are imported</t>
+  </si>
+  <si>
+    <t>share_imported</t>
+  </si>
+  <si>
+    <t>Max total amounts of crop and by-products that are imported</t>
+  </si>
+  <si>
+    <t>max_total_imported</t>
+  </si>
+  <si>
+    <t>kg product</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b val="true"/>
-        <u val="single"/>
+        <b/>
+        <u/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">Maximum contribution of crop to crop product demand for feed</t>
+      <t>Maximum contribution of crop to crop product demand for feed</t>
     </r>
     <r>
       <rPr>
@@ -263,152 +267,155 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">cattle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Semi-natural pastures</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_crop_in_crop_prod</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dairy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Storage and feeding losses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">storage_losses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feeding_losses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ley silage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80% in silo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cederberg &amp; Henriksson (2020)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">60% in silo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No feeding on pasture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bulls</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10% feeding on pasture</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dry concentrates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">??</t>
-  </si>
-  <si>
-    <t xml:space="preserve">for cattle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Statistics Netherlands (2012)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Enteric fermentation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For cattle Ym is calculated from feed ration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">enteric_adj</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adjustment factor for enteric methane emissions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feed nutritional parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">see feed pars sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">General</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">feed_composition</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MJ GE/kg DM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cattle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ME</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MJ ME/kg DM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy in feed used for feed req. calc.: ME for cattle,sheep and horses and NE for pigs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MJ DE/kg DM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">g/kg DM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total fat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">g AAT/kg DM</t>
+    <t>cattle</t>
+  </si>
+  <si>
+    <t>Semi-natural pastures</t>
+  </si>
+  <si>
+    <t>max_crop_in_crop_prod</t>
+  </si>
+  <si>
+    <t>dairy</t>
+  </si>
+  <si>
+    <t>cows</t>
+  </si>
+  <si>
+    <t>Storage and feeding losses</t>
+  </si>
+  <si>
+    <t>storage_losses</t>
+  </si>
+  <si>
+    <t>feeding_losses</t>
+  </si>
+  <si>
+    <t>ley silage</t>
+  </si>
+  <si>
+    <t>80% in silo</t>
+  </si>
+  <si>
+    <t>Cederberg &amp; Henriksson (2020)</t>
+  </si>
+  <si>
+    <t>60% in silo</t>
+  </si>
+  <si>
+    <t>No feeding on pasture</t>
+  </si>
+  <si>
+    <t>bulls</t>
+  </si>
+  <si>
+    <t>10% feeding on pasture</t>
+  </si>
+  <si>
+    <t>dry concentrates</t>
+  </si>
+  <si>
+    <t>??</t>
+  </si>
+  <si>
+    <t>for cattle</t>
+  </si>
+  <si>
+    <t>Statistics Netherlands (2012)</t>
+  </si>
+  <si>
+    <t>Enteric fermentation</t>
+  </si>
+  <si>
+    <t>For cattle Ym is calculated from feed ration</t>
+  </si>
+  <si>
+    <t>enteric_adj</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Adjustment factor for enteric methane emissions</t>
+  </si>
+  <si>
+    <t>Feed nutritional parameters</t>
+  </si>
+  <si>
+    <t>see feed pars sheet</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>GE</t>
+  </si>
+  <si>
+    <t>feed_composition</t>
+  </si>
+  <si>
+    <t>MJ GE/kg DM</t>
+  </si>
+  <si>
+    <t>ASH</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Cattle</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>MJ ME/kg DM</t>
+  </si>
+  <si>
+    <t>Energy in feed used for feed req. calc.: ME for cattle,sheep and horses and NE for pigs</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>MJ DE/kg DM</t>
+  </si>
+  <si>
+    <t>fat</t>
+  </si>
+  <si>
+    <t>g/kg DM</t>
+  </si>
+  <si>
+    <t>Total fat</t>
+  </si>
+  <si>
+    <t>AAT</t>
+  </si>
+  <si>
+    <t>g AAT/kg DM</t>
+  </si>
+  <si>
+    <t>PBV</t>
+  </si>
+  <si>
+    <t>g PBV/kg DM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.00"/>
-    <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="0.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -417,22 +424,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -440,8 +432,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <u val="single"/>
+      <b/>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -476,7 +468,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="4"/>
       <name val="Calibri"/>
@@ -506,7 +498,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -514,113 +506,34 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="18">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -679,60 +592,76 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -764,7 +693,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -788,7 +717,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -848,74 +777,65 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:S1048576"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S138"/>
+  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="20.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="23.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="16.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="38.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="58"/>
+    <col min="6" max="7" width="20.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.5703125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="19.5703125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="20.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="9.7109375" style="1" customWidth="1"/>
+    <col min="13" max="14" width="16.42578125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="10.85546875" style="1" customWidth="1"/>
+    <col min="16" max="16" width="12.7109375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="38.140625" style="1" customWidth="1"/>
+    <col min="18" max="18" width="58" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -971,7 +891,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
@@ -998,11 +918,11 @@
       <c r="R2" s="4"/>
       <c r="S2" s="1"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="N3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="7" t="n">
+      <c r="O3" s="7">
         <v>0</v>
       </c>
       <c r="P3" s="6"/>
@@ -1010,7 +930,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>27</v>
       </c>
@@ -1019,7 +939,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
@@ -1029,11 +949,11 @@
       <c r="N5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="9" t="n">
+      <c r="O5" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1043,11 +963,11 @@
       <c r="N6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O6" s="9" t="n">
+      <c r="O6" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
@@ -1057,11 +977,11 @@
       <c r="N7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O7" s="9" t="n">
+      <c r="O7" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F8" s="1" t="s">
         <v>32</v>
       </c>
@@ -1071,11 +991,11 @@
       <c r="N8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O8" s="9" t="n">
+      <c r="O8" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
@@ -1092,7 +1012,7 @@
       <c r="P9" s="10"/>
       <c r="Q9" s="11"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1102,11 +1022,11 @@
       <c r="N10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O10" s="9" t="n">
+      <c r="O10" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F11" s="1" t="s">
         <v>35</v>
       </c>
@@ -1116,11 +1036,11 @@
       <c r="N11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O11" s="9" t="n">
+      <c r="O11" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="F12" s="1" t="s">
         <v>36</v>
       </c>
@@ -1130,23 +1050,23 @@
       <c r="N12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O12" s="9" t="n">
+      <c r="O12" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="O13" s="9"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>38</v>
       </c>
       <c r="O14" s="9"/>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="O15" s="9"/>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>39</v>
       </c>
@@ -1168,7 +1088,7 @@
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
     </row>
-    <row r="17" s="1" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>40</v>
       </c>
@@ -1176,11 +1096,11 @@
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="O18" s="6" t="n">
+      <c r="O18" s="6">
         <v>0</v>
       </c>
       <c r="P18" s="6" t="s">
@@ -1190,21 +1110,21 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="I19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O19" s="11" t="n">
+      <c r="O19" s="11">
         <v>95</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
@@ -1214,14 +1134,14 @@
       <c r="N20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O20" s="11" t="n">
+      <c r="O20" s="11">
         <v>95</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C21" s="1" t="s">
         <v>44</v>
       </c>
@@ -1231,32 +1151,32 @@
       <c r="N21" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O21" s="11" t="n">
+      <c r="O21" s="11">
         <v>50</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O22" s="11"/>
       <c r="Q22" s="11"/>
     </row>
-    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>45</v>
       </c>
       <c r="O23" s="11"/>
       <c r="Q23" s="11"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="I24" s="1" t="s">
         <v>29</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="O24" s="11" t="n">
+      <c r="O24" s="11">
         <v>5</v>
       </c>
       <c r="P24" s="1" t="s">
@@ -1264,14 +1184,14 @@
       </c>
       <c r="Q24" s="11"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="I25" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="O25" s="11" t="n">
+      <c r="O25" s="11">
         <v>5</v>
       </c>
       <c r="P25" s="1" t="s">
@@ -1279,11 +1199,11 @@
       </c>
       <c r="Q25" s="11"/>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O26" s="11"/>
       <c r="Q26" s="11"/>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>47</v>
       </c>
@@ -1305,11 +1225,11 @@
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N28" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="O28" s="6" t="n">
+      <c r="O28" s="6">
         <v>0</v>
       </c>
       <c r="P28" s="6" t="s">
@@ -1319,7 +1239,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>49</v>
       </c>
@@ -1341,11 +1261,11 @@
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O30" s="6" t="n">
+      <c r="O30" s="6">
         <v>0</v>
       </c>
       <c r="P30" s="6" t="s">
@@ -1355,7 +1275,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C31" s="1" t="s">
         <v>43</v>
       </c>
@@ -1365,13 +1285,13 @@
       <c r="N31" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="O31" s="13" t="n">
+      <c r="O31" s="13">
         <v>100000</v>
       </c>
       <c r="P31" s="13"/>
       <c r="Q31" s="6"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="C32" s="1" t="s">
         <v>43</v>
       </c>
@@ -1381,19 +1301,19 @@
       <c r="N32" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="O32" s="13" t="n">
+      <c r="O32" s="13">
         <v>200000</v>
       </c>
       <c r="P32" s="13"/>
       <c r="Q32" s="6"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
       <c r="Q33" s="6"/>
     </row>
-    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>52</v>
       </c>
@@ -1415,7 +1335,7 @@
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>53</v>
       </c>
@@ -1428,7 +1348,7 @@
       <c r="N36" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="O36" s="10" t="n">
+      <c r="O36" s="10">
         <v>30</v>
       </c>
       <c r="P36" s="1" t="s">
@@ -1436,7 +1356,7 @@
       </c>
       <c r="Q36" s="10"/>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>53</v>
       </c>
@@ -1455,7 +1375,7 @@
       <c r="N37" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="O37" s="10" t="n">
+      <c r="O37" s="10">
         <v>10</v>
       </c>
       <c r="P37" s="1" t="s">
@@ -1463,11 +1383,11 @@
       </c>
       <c r="Q37" s="10"/>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O38" s="11"/>
       <c r="Q38" s="11"/>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>58</v>
       </c>
@@ -1489,11 +1409,11 @@
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N40" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="O40" s="6" t="n">
+      <c r="O40" s="6">
         <v>0</v>
       </c>
       <c r="P40" s="6" t="s">
@@ -1503,11 +1423,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N41" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="O41" s="6" t="n">
+      <c r="O41" s="6">
         <v>0</v>
       </c>
       <c r="P41" s="6" t="s">
@@ -1517,7 +1437,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>53</v>
       </c>
@@ -1533,9 +1453,9 @@
       <c r="N42" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="O42" s="10" t="n">
-        <f aca="false">(0.8*20+0.2*2)</f>
-        <v>16.4</v>
+      <c r="O42" s="10">
+        <f>(0.8*20+0.2*2)</f>
+        <v>16.399999999999999</v>
       </c>
       <c r="P42" s="10" t="s">
         <v>42</v>
@@ -1547,7 +1467,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>53</v>
       </c>
@@ -1557,8 +1477,8 @@
       <c r="N43" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="O43" s="10" t="n">
-        <f aca="false">(0.6*20+0.4*2)</f>
+      <c r="O43" s="10">
+        <f>(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
       <c r="P43" s="10" t="s">
@@ -1571,13 +1491,13 @@
         <v>63</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
       <c r="P44" s="10"/>
       <c r="Q44" s="10"/>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>53</v>
       </c>
@@ -1593,7 +1513,7 @@
       <c r="N45" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O45" s="10" t="n">
+      <c r="O45" s="10">
         <v>5</v>
       </c>
       <c r="P45" s="10" t="s">
@@ -1606,7 +1526,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>53</v>
       </c>
@@ -1619,7 +1539,7 @@
       <c r="N46" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O46" s="10" t="n">
+      <c r="O46" s="10">
         <v>5</v>
       </c>
       <c r="P46" s="10" t="s">
@@ -1632,7 +1552,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>53</v>
       </c>
@@ -1642,8 +1562,8 @@
       <c r="N47" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O47" s="10" t="n">
-        <f aca="false">0.9*5+0.1*15</f>
+      <c r="O47" s="10">
+        <f>0.9*5+0.1*15</f>
         <v>6</v>
       </c>
       <c r="P47" s="10" t="s">
@@ -1656,13 +1576,13 @@
         <v>63</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
       <c r="P48" s="10"/>
       <c r="Q48" s="10"/>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="11"/>
       <c r="G49" s="1" t="s">
         <v>68</v>
@@ -1675,7 +1595,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="11"/>
       <c r="G50" s="1" t="s">
         <v>68</v>
@@ -1683,7 +1603,7 @@
       <c r="N50" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O50" s="10" t="n">
+      <c r="O50" s="10">
         <v>2</v>
       </c>
       <c r="P50" s="10" t="s">
@@ -1696,14 +1616,14 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="11"/>
       <c r="N51" s="10"/>
       <c r="O51" s="10"/>
       <c r="P51" s="10"/>
       <c r="Q51" s="11"/>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>72</v>
       </c>
@@ -1725,7 +1645,7 @@
       <c r="Q52" s="4"/>
       <c r="R52" s="4"/>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -1734,15 +1654,15 @@
         <v>73</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O54" s="10"/>
       <c r="Q54" s="11"/>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N55" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="O55" s="10" t="n">
+      <c r="O55" s="10">
         <v>1</v>
       </c>
       <c r="P55" s="10" t="s">
@@ -1753,11 +1673,11 @@
       </c>
       <c r="R55" s="10"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O56" s="11"/>
       <c r="Q56" s="11"/>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>77</v>
       </c>
@@ -1781,12 +1701,12 @@
       </c>
       <c r="R57" s="4"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A58" s="8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F59" s="1" t="s">
         <v>28</v>
       </c>
@@ -1796,14 +1716,14 @@
       <c r="N59" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O59" s="14" t="n">
-        <v>17.3169484</v>
+      <c r="O59" s="14">
+        <v>17.316948400000001</v>
       </c>
       <c r="P59" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F60" s="1" t="s">
         <v>30</v>
       </c>
@@ -1813,11 +1733,11 @@
       <c r="N60" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O60" s="14" t="n">
+      <c r="O60" s="14">
         <v>17.150216</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F61" s="1" t="s">
         <v>31</v>
       </c>
@@ -1827,11 +1747,11 @@
       <c r="N61" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O61" s="14" t="n">
-        <v>17.41143707</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O61" s="14">
+        <v>17.411437070000002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F62" s="1" t="s">
         <v>32</v>
       </c>
@@ -1841,11 +1761,11 @@
       <c r="N62" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O62" s="14" t="n">
-        <v>18.2100232</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O62" s="14">
+        <v>18.210023199999998</v>
+      </c>
+    </row>
+    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F63" s="1" t="s">
         <v>34</v>
       </c>
@@ -1855,11 +1775,11 @@
       <c r="N63" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O63" s="14" t="n">
-        <v>19.589488</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O63" s="14">
+        <v>19.589487999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
       <c r="F64" s="1" t="s">
         <v>35</v>
       </c>
@@ -1869,11 +1789,11 @@
       <c r="N64" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O64" s="14" t="n">
+      <c r="O64" s="14">
         <v>19.4920008</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F65" s="1" t="s">
         <v>36</v>
       </c>
@@ -1883,14 +1803,14 @@
       <c r="N65" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O65" s="14" t="n">
-        <v>18.194124</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O65" s="14">
+        <v>18.194123999999999</v>
+      </c>
+    </row>
+    <row r="66" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O66" s="14"/>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F67" s="1" t="s">
         <v>28</v>
       </c>
@@ -1900,11 +1820,11 @@
       <c r="N67" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O67" s="16" t="n">
+      <c r="O67" s="16">
         <v>7.55</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F68" s="1" t="s">
         <v>30</v>
       </c>
@@ -1914,11 +1834,11 @@
       <c r="N68" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O68" s="16" t="n">
+      <c r="O68" s="16">
         <v>7.8</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F69" s="1" t="s">
         <v>31</v>
       </c>
@@ -1928,11 +1848,11 @@
       <c r="N69" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O69" s="16" t="n">
-        <v>6.566666667</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O69" s="16">
+        <v>6.5666666669999998</v>
+      </c>
+    </row>
+    <row r="70" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F70" s="1" t="s">
         <v>32</v>
       </c>
@@ -1942,11 +1862,11 @@
       <c r="N70" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O70" s="16" t="n">
+      <c r="O70" s="16">
         <v>1.8</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F71" s="1" t="s">
         <v>34</v>
       </c>
@@ -1956,11 +1876,11 @@
       <c r="N71" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O71" s="16" t="n">
+      <c r="O71" s="16">
         <v>7.15</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F72" s="1" t="s">
         <v>35</v>
       </c>
@@ -1970,11 +1890,11 @@
       <c r="N72" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O72" s="16" t="n">
+      <c r="O72" s="16">
         <v>7.7</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F73" s="1" t="s">
         <v>36</v>
       </c>
@@ -1984,14 +1904,14 @@
       <c r="N73" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O73" s="16" t="n">
+      <c r="O73" s="16">
         <v>5.9</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O74" s="16"/>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F75" s="1" t="s">
         <v>28</v>
       </c>
@@ -2001,11 +1921,11 @@
       <c r="N75" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O75" s="16" t="n">
-        <v>2.424</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O75" s="16">
+        <v>2.4239999999999999</v>
+      </c>
+    </row>
+    <row r="76" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F76" s="1" t="s">
         <v>30</v>
       </c>
@@ -2015,11 +1935,11 @@
       <c r="N76" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O76" s="16" t="n">
-        <v>2.128</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O76" s="16">
+        <v>2.1280000000000001</v>
+      </c>
+    </row>
+    <row r="77" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F77" s="1" t="s">
         <v>31</v>
       </c>
@@ -2029,11 +1949,11 @@
       <c r="N77" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O77" s="16" t="n">
+      <c r="O77" s="16">
         <v>2.246666667</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F78" s="1" t="s">
         <v>32</v>
       </c>
@@ -2043,11 +1963,11 @@
       <c r="N78" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O78" s="16" t="n">
-        <v>1.936</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O78" s="16">
+        <v>1.9359999999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F79" s="1" t="s">
         <v>34</v>
       </c>
@@ -2057,11 +1977,11 @@
       <c r="N79" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O79" s="16" t="n">
-        <v>8.208</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O79" s="16">
+        <v>8.2080000000000002</v>
+      </c>
+    </row>
+    <row r="80" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F80" s="1" t="s">
         <v>35</v>
       </c>
@@ -2071,11 +1991,11 @@
       <c r="N80" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O80" s="16" t="n">
-        <v>6.152</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O80" s="16">
+        <v>6.1520000000000001</v>
+      </c>
+    </row>
+    <row r="81" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F81" s="1" t="s">
         <v>36</v>
       </c>
@@ -2085,14 +2005,14 @@
       <c r="N81" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O81" s="16" t="n">
+      <c r="O81" s="16">
         <v>2.64</v>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O82" s="16"/>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F83" s="1" t="s">
         <v>28</v>
       </c>
@@ -2102,11 +2022,11 @@
       <c r="N83" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O83" s="16" t="n">
-        <v>0.28</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O83" s="16">
+        <v>0.28000000000000003</v>
+      </c>
+    </row>
+    <row r="84" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F84" s="1" t="s">
         <v>30</v>
       </c>
@@ -2116,11 +2036,11 @@
       <c r="N84" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O84" s="16" t="n">
+      <c r="O84" s="16">
         <v>0.27</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F85" s="1" t="s">
         <v>31</v>
       </c>
@@ -2130,11 +2050,11 @@
       <c r="N85" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O85" s="16" t="n">
+      <c r="O85" s="16">
         <v>0.27</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F86" s="1" t="s">
         <v>32</v>
       </c>
@@ -2144,11 +2064,11 @@
       <c r="N86" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O86" s="16" t="n">
-        <v>0.345</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O86" s="16">
+        <v>0.34499999999999997</v>
+      </c>
+    </row>
+    <row r="87" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F87" s="1" t="s">
         <v>34</v>
       </c>
@@ -2158,11 +2078,11 @@
       <c r="N87" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O87" s="16" t="n">
-        <v>0.715</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O87" s="16">
+        <v>0.71499999999999997</v>
+      </c>
+    </row>
+    <row r="88" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F88" s="1" t="s">
         <v>35</v>
       </c>
@@ -2172,11 +2092,11 @@
       <c r="N88" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O88" s="16" t="n">
-        <v>1.245</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O88" s="16">
+        <v>1.2450000000000001</v>
+      </c>
+    </row>
+    <row r="89" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F89" s="1" t="s">
         <v>36</v>
       </c>
@@ -2186,14 +2106,14 @@
       <c r="N89" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O89" s="16" t="n">
-        <v>1.195</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O89" s="16">
+        <v>1.1950000000000001</v>
+      </c>
+    </row>
+    <row r="90" spans="6:15" x14ac:dyDescent="0.25">
       <c r="O90" s="16"/>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F91" s="1" t="s">
         <v>28</v>
       </c>
@@ -2203,11 +2123,11 @@
       <c r="N91" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O91" s="16" t="n">
-        <v>2.425</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O91" s="16">
+        <v>2.4249999999999998</v>
+      </c>
+    </row>
+    <row r="92" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F92" s="1" t="s">
         <v>30</v>
       </c>
@@ -2217,11 +2137,11 @@
       <c r="N92" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O92" s="16" t="n">
+      <c r="O92" s="16">
         <v>2.34</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F93" s="1" t="s">
         <v>31</v>
       </c>
@@ -2231,11 +2151,11 @@
       <c r="N93" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O93" s="16" t="n">
+      <c r="O93" s="16">
         <v>2.34</v>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F94" s="1" t="s">
         <v>32</v>
       </c>
@@ -2245,11 +2165,11 @@
       <c r="N94" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O94" s="16" t="n">
-        <v>0.525</v>
-      </c>
-    </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O94" s="16">
+        <v>0.52500000000000002</v>
+      </c>
+    </row>
+    <row r="95" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F95" s="1" t="s">
         <v>34</v>
       </c>
@@ -2259,11 +2179,11 @@
       <c r="N95" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O95" s="16" t="n">
+      <c r="O95" s="16">
         <v>2.35</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F96" s="1" t="s">
         <v>35</v>
       </c>
@@ -2273,11 +2193,11 @@
       <c r="N96" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O96" s="16" t="n">
+      <c r="O96" s="16">
         <v>1.55</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F97" s="1" t="s">
         <v>36</v>
       </c>
@@ -2287,20 +2207,20 @@
       <c r="N97" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O97" s="16" t="n">
+      <c r="O97" s="16">
         <v>1.35</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
       <c r="O98" s="14"/>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="8" t="s">
         <v>87</v>
       </c>
       <c r="O99" s="14"/>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>53</v>
       </c>
@@ -2313,7 +2233,7 @@
       <c r="N100" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O100" s="14" t="n">
+      <c r="O100" s="14">
         <v>11.3</v>
       </c>
       <c r="P100" s="1" t="s">
@@ -2323,7 +2243,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>53</v>
       </c>
@@ -2336,12 +2256,12 @@
       <c r="N101" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O101" s="14" t="n">
+      <c r="O101" s="14">
         <v>10.1</v>
       </c>
       <c r="Q101" s="10"/>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>53</v>
       </c>
@@ -2354,12 +2274,12 @@
       <c r="N102" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O102" s="14" t="n">
-        <v>9.941666667</v>
+      <c r="O102" s="14">
+        <v>9.9416666669999998</v>
       </c>
       <c r="Q102" s="10"/>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>53</v>
       </c>
@@ -2372,12 +2292,12 @@
       <c r="N103" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O103" s="14" t="n">
+      <c r="O103" s="14">
         <v>14.1</v>
       </c>
       <c r="Q103" s="10"/>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>53</v>
       </c>
@@ -2390,12 +2310,12 @@
       <c r="N104" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O104" s="14" t="n">
+      <c r="O104" s="14">
         <v>14.6</v>
       </c>
       <c r="Q104" s="10"/>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>53</v>
       </c>
@@ -2408,12 +2328,12 @@
       <c r="N105" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O105" s="14" t="n">
+      <c r="O105" s="14">
         <v>12.2</v>
       </c>
       <c r="Q105" s="10"/>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>53</v>
       </c>
@@ -2426,16 +2346,16 @@
       <c r="N106" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O106" s="14" t="n">
+      <c r="O106" s="14">
         <v>11</v>
       </c>
       <c r="Q106" s="10"/>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
       <c r="O107" s="17"/>
       <c r="Q107" s="10"/>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>53</v>
       </c>
@@ -2448,7 +2368,7 @@
       <c r="N108" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O108" s="14" t="n">
+      <c r="O108" s="14">
         <v>13.35</v>
       </c>
       <c r="P108" s="1" t="s">
@@ -2456,7 +2376,7 @@
       </c>
       <c r="Q108" s="11"/>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>53</v>
       </c>
@@ -2469,12 +2389,12 @@
       <c r="N109" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O109" s="14" t="n">
+      <c r="O109" s="14">
         <v>11.9</v>
       </c>
       <c r="Q109" s="11"/>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>53</v>
       </c>
@@ -2487,12 +2407,12 @@
       <c r="N110" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O110" s="14" t="n">
+      <c r="O110" s="14">
         <v>12.4</v>
       </c>
       <c r="Q110" s="11"/>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>53</v>
       </c>
@@ -2505,12 +2425,12 @@
       <c r="N111" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O111" s="14" t="n">
+      <c r="O111" s="14">
         <v>16</v>
       </c>
       <c r="Q111" s="11"/>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>53</v>
       </c>
@@ -2523,12 +2443,12 @@
       <c r="N112" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O112" s="14" t="n">
+      <c r="O112" s="14">
         <v>17.8</v>
       </c>
       <c r="Q112" s="11"/>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>53</v>
       </c>
@@ -2541,12 +2461,12 @@
       <c r="N113" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O113" s="14" t="n">
+      <c r="O113" s="14">
         <v>14.6</v>
       </c>
       <c r="Q113" s="11"/>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>53</v>
       </c>
@@ -2559,16 +2479,16 @@
       <c r="N114" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O114" s="14" t="n">
+      <c r="O114" s="14">
         <v>12.7</v>
       </c>
       <c r="Q114" s="11"/>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
       <c r="O115" s="17"/>
       <c r="Q115" s="11"/>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>53</v>
       </c>
@@ -2581,7 +2501,7 @@
       <c r="N116" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O116" s="14" t="n">
+      <c r="O116" s="14">
         <v>20</v>
       </c>
       <c r="P116" s="1" t="s">
@@ -2591,7 +2511,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>53</v>
       </c>
@@ -2604,12 +2524,12 @@
       <c r="N117" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O117" s="14" t="n">
+      <c r="O117" s="14">
         <v>20</v>
       </c>
       <c r="Q117" s="10"/>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>53</v>
       </c>
@@ -2622,12 +2542,12 @@
       <c r="N118" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O118" s="14" t="n">
+      <c r="O118" s="14">
         <v>20</v>
       </c>
       <c r="Q118" s="11"/>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>53</v>
       </c>
@@ -2640,11 +2560,11 @@
       <c r="N119" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O119" s="14" t="n">
+      <c r="O119" s="14">
         <v>25</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>53</v>
       </c>
@@ -2657,12 +2577,12 @@
       <c r="N120" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O120" s="14" t="n">
+      <c r="O120" s="14">
         <v>10</v>
       </c>
       <c r="Q120" s="10"/>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>53</v>
       </c>
@@ -2675,12 +2595,12 @@
       <c r="N121" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O121" s="14" t="n">
+      <c r="O121" s="14">
         <v>46</v>
       </c>
       <c r="Q121" s="11"/>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>53</v>
       </c>
@@ -2693,15 +2613,15 @@
       <c r="N122" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O122" s="14" t="n">
+      <c r="O122" s="14">
         <v>45</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
       <c r="O123" s="10"/>
       <c r="Q123" s="10"/>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>53</v>
       </c>
@@ -2714,7 +2634,7 @@
       <c r="N124" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O124" s="14" t="n">
+      <c r="O124" s="14">
         <v>72</v>
       </c>
       <c r="P124" s="1" t="s">
@@ -2722,7 +2642,7 @@
       </c>
       <c r="Q124" s="11"/>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>53</v>
       </c>
@@ -2736,14 +2656,14 @@
       <c r="N125" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O125" s="14" t="n">
+      <c r="O125" s="14">
         <v>69</v>
       </c>
       <c r="P125" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>53</v>
       </c>
@@ -2756,7 +2676,7 @@
       <c r="N126" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O126" s="14" t="n">
+      <c r="O126" s="14">
         <v>74.3333333333333</v>
       </c>
       <c r="P126" s="1" t="s">
@@ -2764,7 +2684,7 @@
       </c>
       <c r="Q126" s="10"/>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>53</v>
       </c>
@@ -2777,14 +2697,14 @@
       <c r="N127" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O127" s="14" t="n">
+      <c r="O127" s="14">
         <v>95</v>
       </c>
       <c r="P127" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>53</v>
       </c>
@@ -2797,14 +2717,14 @@
       <c r="N128" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O128" s="14" t="n">
+      <c r="O128" s="14">
         <v>182</v>
       </c>
       <c r="P128" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>53</v>
       </c>
@@ -2817,14 +2737,14 @@
       <c r="N129" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O129" s="14" t="n">
+      <c r="O129" s="14">
         <v>221</v>
       </c>
       <c r="P129" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>53</v>
       </c>
@@ -2837,22 +2757,155 @@
       <c r="N130" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O130" s="14" t="n">
+      <c r="O130" s="14">
         <v>73</v>
       </c>
       <c r="P130" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A132" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M132" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N132" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O132">
+        <v>26.5</v>
+      </c>
+      <c r="P132" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A133" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="M133" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N133" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O133">
+        <v>14</v>
+      </c>
+      <c r="P133" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A134" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M134" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N134" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O134">
+        <v>12.25</v>
+      </c>
+      <c r="P134" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A135" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="M135" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N135" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O135">
+        <v>-33</v>
+      </c>
+      <c r="P135" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A136" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M136" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N136" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O136">
+        <v>261</v>
+      </c>
+      <c r="P136" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A137" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="M137" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N137" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O137">
+        <v>79</v>
+      </c>
+      <c r="P137" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A138" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="M138" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="N138" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="O138">
+        <v>36</v>
+      </c>
+      <c r="P138" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Bugfix: mismatch in units for fat Contents was in g/kg DM, limit in percentage
</commit_message>
<xml_diff>
--- a/mini/data/default/FeedMgmt.xlsx
+++ b/mini/data/default/FeedMgmt.xlsx
@@ -1,21 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\mini\data\default\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="references" sheetId="1" r:id="rId1"/>
-    <sheet name="default" sheetId="2" r:id="rId2"/>
+    <sheet name="references" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="default" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -27,124 +23,124 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="100">
   <si>
-    <t>Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
-  </si>
-  <si>
-    <t>Cederberg, C. &amp; Henriksson, M. (2020). Gräsmarkernas användning i jordbruket</t>
-  </si>
-  <si>
-    <t>Hessle, A. &amp; Danielsson, R. (2023) Number of cattle required to obtain good ecological status in Swedish grasslands and livestock’s methane emissions. Swedish University of Agricultural Sciences. Department of Animal Environment and Health. Section of Production systems</t>
-  </si>
-  <si>
-    <t>Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
-  </si>
-  <si>
-    <t>f_species</t>
-  </si>
-  <si>
-    <t>f_breed</t>
-  </si>
-  <si>
-    <t>f_prod_system</t>
-  </si>
-  <si>
-    <t>f_sub_system</t>
-  </si>
-  <si>
-    <t>f_animal</t>
-  </si>
-  <si>
-    <t>f_feed</t>
-  </si>
-  <si>
-    <t>f_feed_group:feed</t>
-  </si>
-  <si>
-    <t>f_crop_group</t>
-  </si>
-  <si>
-    <t>f_crop_prod</t>
-  </si>
-  <si>
-    <t>f_by_prod</t>
-  </si>
-  <si>
-    <t>f_crop_resid</t>
-  </si>
-  <si>
-    <t>f_region</t>
-  </si>
-  <si>
-    <t>f_feed_par</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>unit</t>
-  </si>
-  <si>
-    <t>description</t>
-  </si>
-  <si>
-    <t>source</t>
-  </si>
-  <si>
-    <t>Conversion factors: Feeds --&gt; crop products, by-products or crop residues</t>
-  </si>
-  <si>
-    <t>kg product/kg DM feed</t>
-  </si>
-  <si>
-    <t>need to align with DM in products and by-products</t>
-  </si>
-  <si>
-    <t>feed_to_prod</t>
-  </si>
-  <si>
-    <t>fallback</t>
-  </si>
-  <si>
-    <t>Crop products</t>
-  </si>
-  <si>
-    <t>ley silage, 1st cut</t>
-  </si>
-  <si>
-    <t>fodder</t>
-  </si>
-  <si>
-    <t>ley silage, regrowth</t>
-  </si>
-  <si>
-    <t>grazing</t>
-  </si>
-  <si>
-    <t>wheat</t>
-  </si>
-  <si>
-    <t>By-products</t>
-  </si>
-  <si>
-    <t>soybean meal</t>
-  </si>
-  <si>
-    <t>rapeseed meal</t>
-  </si>
-  <si>
-    <t>wheat bran</t>
-  </si>
-  <si>
-    <t>milling by-products from wheat, barley or rye</t>
-  </si>
-  <si>
-    <t>Crop residues</t>
-  </si>
-  <si>
-    <t>Parameters to constrain regional feed supply</t>
+    <t xml:space="preserve">Statistics Netherlands (2012) Standardised calculation methods for animal manure and nutrients. Standard data 1990–2008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cederberg, C. &amp; Henriksson, M. (2020). Gräsmarkernas användning i jordbruket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hessle, A. &amp; Danielsson, R. (2023) Number of cattle required to obtain good ecological status in Swedish grasslands and livestock’s methane emissions. Swedish University of Agricultural Sciences. Department of Animal Environment and Health. Section of Production systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ahlgren, S., Behaderovic, D., Wirsenius, S., Carlsson, A., Hessle, A. Toräng, P., Seeman, A., den Braver, T. &amp;  et al. Kvarnbäck, O. (2022) Miljöpåverkan av svensk nöt- och lammköttsproduktion. RISE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_species</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_breed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_prod_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_sub_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_animal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_feed_group:feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_crop_group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_crop_prod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_by_prod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_crop_resid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_feed_par</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversion factors: Feeds --&gt; crop products, by-products or crop residues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg product/kg DM feed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">need to align with DM in products and by-products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feed_to_prod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fallback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crop products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ley silage, 1st cut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fodder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ley silage, regrowth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grazing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wheat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">By-products</t>
+  </si>
+  <si>
+    <t xml:space="preserve">soybean meal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rapeseed meal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wheat bran</t>
+  </si>
+  <si>
+    <t xml:space="preserve">milling by-products from wheat, barley or rye</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crop residues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parameters to constrain regional feed supply</t>
   </si>
   <si>
     <r>
@@ -155,11 +151,11 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t>The parameter</t>
+      <t xml:space="preserve">The parameter</t>
     </r>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color theme="4"/>
         <rFont val="Calibri"/>
@@ -180,16 +176,16 @@
     </r>
   </si>
   <si>
-    <t>share_regional</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>conventional</t>
-  </si>
-  <si>
-    <t>organic</t>
+    <t xml:space="preserve">share_regional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">conventional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">organic</t>
   </si>
   <si>
     <r>
@@ -204,14 +200,14 @@
     </r>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color theme="4"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t>max_overproduction</t>
+      <t xml:space="preserve">max_overproduction</t>
     </r>
     <r>
       <rPr>
@@ -225,35 +221,35 @@
     </r>
   </si>
   <si>
-    <t>max_overproduction</t>
-  </si>
-  <si>
-    <t>Share of crop and by-products that are imported</t>
-  </si>
-  <si>
-    <t>share_imported</t>
-  </si>
-  <si>
-    <t>Max total amounts of crop and by-products that are imported</t>
-  </si>
-  <si>
-    <t>max_total_imported</t>
-  </si>
-  <si>
-    <t>kg product</t>
+    <t xml:space="preserve">max_overproduction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of crop and by-products that are imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">share_imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max total amounts of crop and by-products that are imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_total_imported</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg product</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
-        <u/>
+        <b val="true"/>
+        <u val="single"/>
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Calibri"/>
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t>Maximum contribution of crop to crop product demand for feed</t>
+      <t xml:space="preserve">Maximum contribution of crop to crop product demand for feed</t>
     </r>
     <r>
       <rPr>
@@ -267,155 +263,158 @@
     </r>
   </si>
   <si>
-    <t>cattle</t>
-  </si>
-  <si>
-    <t>Semi-natural pastures</t>
-  </si>
-  <si>
-    <t>max_crop_in_crop_prod</t>
-  </si>
-  <si>
-    <t>dairy</t>
-  </si>
-  <si>
-    <t>cows</t>
-  </si>
-  <si>
-    <t>Storage and feeding losses</t>
-  </si>
-  <si>
-    <t>storage_losses</t>
-  </si>
-  <si>
-    <t>feeding_losses</t>
-  </si>
-  <si>
-    <t>ley silage</t>
-  </si>
-  <si>
-    <t>80% in silo</t>
-  </si>
-  <si>
-    <t>Cederberg &amp; Henriksson (2020)</t>
-  </si>
-  <si>
-    <t>60% in silo</t>
-  </si>
-  <si>
-    <t>No feeding on pasture</t>
-  </si>
-  <si>
-    <t>bulls</t>
-  </si>
-  <si>
-    <t>10% feeding on pasture</t>
-  </si>
-  <si>
-    <t>dry concentrates</t>
-  </si>
-  <si>
-    <t>??</t>
-  </si>
-  <si>
-    <t>for cattle</t>
-  </si>
-  <si>
-    <t>Statistics Netherlands (2012)</t>
-  </si>
-  <si>
-    <t>Enteric fermentation</t>
-  </si>
-  <si>
-    <t>For cattle Ym is calculated from feed ration</t>
-  </si>
-  <si>
-    <t>enteric_adj</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Adjustment factor for enteric methane emissions</t>
-  </si>
-  <si>
-    <t>Feed nutritional parameters</t>
-  </si>
-  <si>
-    <t>see feed pars sheet</t>
-  </si>
-  <si>
-    <t>General</t>
-  </si>
-  <si>
-    <t>GE</t>
-  </si>
-  <si>
-    <t>feed_composition</t>
-  </si>
-  <si>
-    <t>MJ GE/kg DM</t>
-  </si>
-  <si>
-    <t>ASH</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>Cattle</t>
-  </si>
-  <si>
-    <t>ME</t>
-  </si>
-  <si>
-    <t>MJ ME/kg DM</t>
-  </si>
-  <si>
-    <t>Energy in feed used for feed req. calc.: ME for cattle,sheep and horses and NE for pigs</t>
-  </si>
-  <si>
-    <t>DE</t>
-  </si>
-  <si>
-    <t>MJ DE/kg DM</t>
-  </si>
-  <si>
-    <t>fat</t>
-  </si>
-  <si>
-    <t>g/kg DM</t>
-  </si>
-  <si>
-    <t>Total fat</t>
-  </si>
-  <si>
-    <t>AAT</t>
-  </si>
-  <si>
-    <t>g AAT/kg DM</t>
-  </si>
-  <si>
-    <t>PBV</t>
-  </si>
-  <si>
-    <t>g PBV/kg DM</t>
+    <t xml:space="preserve">cattle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Semi-natural pastures</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max_crop_in_crop_prod</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dairy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storage and feeding losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">storage_losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feeding_losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ley silage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80% in silo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cederberg &amp; Henriksson (2020)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60% in silo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No feeding on pasture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bulls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% feeding on pasture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dry concentrates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">??</t>
+  </si>
+  <si>
+    <t xml:space="preserve">for cattle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statistics Netherlands (2012)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enteric fermentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For cattle Ym is calculated from feed ration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enteric_adj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjustment factor for enteric methane emissions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Feed nutritional parameters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see feed pars sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">feed_composition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MJ GE/kg DM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cattle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MJ ME/kg DM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy in feed used for feed req. calc.: ME for cattle,sheep and horses and NE for pigs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MJ DE/kg DM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g/kg DM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total fat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g AAT/kg DM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PBV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g PBV/kg DM</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -424,7 +423,22 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -432,8 +446,8 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
-      <u/>
+      <b val="true"/>
+      <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -468,7 +482,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <b val="true"/>
       <sz val="11"/>
       <color theme="4"/>
       <name val="Calibri"/>
@@ -498,7 +512,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -506,34 +520,113 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="18">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -592,76 +685,60 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -693,7 +770,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -717,7 +794,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -777,65 +854,75 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S138"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:S145"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="6" max="7" width="20.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="19.5703125" style="1" customWidth="1"/>
-    <col min="10" max="11" width="20.140625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="9.7109375" style="1" customWidth="1"/>
-    <col min="13" max="14" width="16.42578125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" style="1" customWidth="1"/>
-    <col min="16" max="16" width="12.7109375" style="1" customWidth="1"/>
-    <col min="17" max="17" width="38.140625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="58" style="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="7" min="7" style="1" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="23.57"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="9" min="9" style="1" width="19.57"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="11" min="10" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="16.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="10.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="12.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="38.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="58"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -891,7 +978,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
@@ -918,11 +1005,11 @@
       <c r="R2" s="4"/>
       <c r="S2" s="1"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N3" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="7">
+      <c r="O3" s="7" t="n">
         <v>0</v>
       </c>
       <c r="P3" s="6"/>
@@ -930,7 +1017,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
         <v>27</v>
       </c>
@@ -939,7 +1026,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F5" s="1" t="s">
         <v>28</v>
       </c>
@@ -949,11 +1036,11 @@
       <c r="N5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F6" s="1" t="s">
         <v>30</v>
       </c>
@@ -963,11 +1050,11 @@
       <c r="N6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O6" s="9">
+      <c r="O6" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
@@ -977,11 +1064,11 @@
       <c r="N7" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O7" s="9">
+      <c r="O7" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F8" s="1" t="s">
         <v>32</v>
       </c>
@@ -991,11 +1078,11 @@
       <c r="N8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O8" s="9">
+      <c r="O8" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
         <v>33</v>
       </c>
@@ -1012,7 +1099,7 @@
       <c r="P9" s="10"/>
       <c r="Q9" s="11"/>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F10" s="1" t="s">
         <v>34</v>
       </c>
@@ -1022,11 +1109,11 @@
       <c r="N10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O10" s="9">
+      <c r="O10" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F11" s="1" t="s">
         <v>35</v>
       </c>
@@ -1036,11 +1123,11 @@
       <c r="N11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O11" s="9">
+      <c r="O11" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F12" s="1" t="s">
         <v>36</v>
       </c>
@@ -1050,23 +1137,23 @@
       <c r="N12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="O12" s="9">
+      <c r="O12" s="9" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O13" s="9"/>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
         <v>38</v>
       </c>
       <c r="O14" s="9"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O15" s="9"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
         <v>39</v>
       </c>
@@ -1088,7 +1175,7 @@
       <c r="Q16" s="4"/>
       <c r="R16" s="4"/>
     </row>
-    <row r="17" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" s="1" customFormat="true" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
         <v>40</v>
       </c>
@@ -1096,11 +1183,11 @@
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N18" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="O18" s="6">
+      <c r="O18" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P18" s="6" t="s">
@@ -1110,21 +1197,21 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O19" s="11">
+      <c r="O19" s="11" t="n">
         <v>95</v>
       </c>
       <c r="P19" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="1" t="s">
         <v>43</v>
       </c>
@@ -1134,14 +1221,14 @@
       <c r="N20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O20" s="11">
+      <c r="O20" s="11" t="n">
         <v>95</v>
       </c>
       <c r="P20" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="1" t="s">
         <v>44</v>
       </c>
@@ -1151,32 +1238,32 @@
       <c r="N21" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="O21" s="11">
+      <c r="O21" s="11" t="n">
         <v>50</v>
       </c>
       <c r="P21" s="1" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O22" s="11"/>
       <c r="Q22" s="11"/>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
         <v>45</v>
       </c>
       <c r="O23" s="11"/>
       <c r="Q23" s="11"/>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I24" s="1" t="s">
         <v>29</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="O24" s="11">
+      <c r="O24" s="11" t="n">
         <v>5</v>
       </c>
       <c r="P24" s="1" t="s">
@@ -1184,14 +1271,14 @@
       </c>
       <c r="Q24" s="11"/>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I25" s="1" t="s">
         <v>31</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="O25" s="11">
+      <c r="O25" s="11" t="n">
         <v>5</v>
       </c>
       <c r="P25" s="1" t="s">
@@ -1199,11 +1286,11 @@
       </c>
       <c r="Q25" s="11"/>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O26" s="11"/>
       <c r="Q26" s="11"/>
     </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
         <v>47</v>
       </c>
@@ -1225,11 +1312,11 @@
       <c r="Q27" s="4"/>
       <c r="R27" s="4"/>
     </row>
-    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N28" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="O28" s="6">
+      <c r="O28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P28" s="6" t="s">
@@ -1239,7 +1326,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
         <v>49</v>
       </c>
@@ -1261,11 +1348,11 @@
       <c r="Q29" s="4"/>
       <c r="R29" s="4"/>
     </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N30" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="O30" s="6">
+      <c r="O30" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P30" s="6" t="s">
@@ -1275,7 +1362,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C31" s="1" t="s">
         <v>43</v>
       </c>
@@ -1285,13 +1372,13 @@
       <c r="N31" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="O31" s="13">
+      <c r="O31" s="13" t="n">
         <v>100000</v>
       </c>
       <c r="P31" s="13"/>
       <c r="Q31" s="6"/>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C32" s="1" t="s">
         <v>43</v>
       </c>
@@ -1301,19 +1388,19 @@
       <c r="N32" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="O32" s="13">
+      <c r="O32" s="13" t="n">
         <v>200000</v>
       </c>
       <c r="P32" s="13"/>
       <c r="Q32" s="6"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N33" s="6"/>
       <c r="O33" s="6"/>
       <c r="P33" s="6"/>
       <c r="Q33" s="6"/>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
         <v>52</v>
       </c>
@@ -1335,7 +1422,7 @@
       <c r="Q34" s="4"/>
       <c r="R34" s="4"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
         <v>53</v>
       </c>
@@ -1348,7 +1435,7 @@
       <c r="N36" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="O36" s="10">
+      <c r="O36" s="10" t="n">
         <v>30</v>
       </c>
       <c r="P36" s="1" t="s">
@@ -1356,7 +1443,7 @@
       </c>
       <c r="Q36" s="10"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
         <v>53</v>
       </c>
@@ -1375,7 +1462,7 @@
       <c r="N37" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="O37" s="10">
+      <c r="O37" s="10" t="n">
         <v>10</v>
       </c>
       <c r="P37" s="1" t="s">
@@ -1383,11 +1470,11 @@
       </c>
       <c r="Q37" s="10"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O38" s="11"/>
       <c r="Q38" s="11"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
         <v>58</v>
       </c>
@@ -1409,11 +1496,11 @@
       <c r="Q39" s="4"/>
       <c r="R39" s="4"/>
     </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N40" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="O40" s="6">
+      <c r="O40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P40" s="6" t="s">
@@ -1423,11 +1510,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N41" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="O41" s="6">
+      <c r="O41" s="6" t="n">
         <v>0</v>
       </c>
       <c r="P41" s="6" t="s">
@@ -1437,7 +1524,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
         <v>53</v>
       </c>
@@ -1453,9 +1540,9 @@
       <c r="N42" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="O42" s="10">
-        <f>(0.8*20+0.2*2)</f>
-        <v>16.399999999999999</v>
+      <c r="O42" s="10" t="n">
+        <f aca="false">(0.8*20+0.2*2)</f>
+        <v>16.4</v>
       </c>
       <c r="P42" s="10" t="s">
         <v>42</v>
@@ -1467,7 +1554,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
         <v>53</v>
       </c>
@@ -1477,8 +1564,8 @@
       <c r="N43" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="O43" s="10">
-        <f>(0.6*20+0.4*2)</f>
+      <c r="O43" s="10" t="n">
+        <f aca="false">(0.6*20+0.4*2)</f>
         <v>12.8</v>
       </c>
       <c r="P43" s="10" t="s">
@@ -1491,13 +1578,13 @@
         <v>63</v>
       </c>
     </row>
-    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N44" s="10"/>
       <c r="O44" s="10"/>
       <c r="P44" s="10"/>
       <c r="Q44" s="10"/>
     </row>
-    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
         <v>53</v>
       </c>
@@ -1513,7 +1600,7 @@
       <c r="N45" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O45" s="10">
+      <c r="O45" s="10" t="n">
         <v>5</v>
       </c>
       <c r="P45" s="10" t="s">
@@ -1526,7 +1613,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
         <v>53</v>
       </c>
@@ -1539,7 +1626,7 @@
       <c r="N46" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O46" s="10">
+      <c r="O46" s="10" t="n">
         <v>5</v>
       </c>
       <c r="P46" s="10" t="s">
@@ -1552,7 +1639,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
         <v>53</v>
       </c>
@@ -1562,8 +1649,8 @@
       <c r="N47" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O47" s="10">
-        <f>0.9*5+0.1*15</f>
+      <c r="O47" s="10" t="n">
+        <f aca="false">0.9*5+0.1*15</f>
         <v>6</v>
       </c>
       <c r="P47" s="10" t="s">
@@ -1576,13 +1663,13 @@
         <v>63</v>
       </c>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
       <c r="P48" s="10"/>
       <c r="Q48" s="10"/>
     </row>
-    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="11"/>
       <c r="G49" s="1" t="s">
         <v>68</v>
@@ -1595,7 +1682,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11"/>
       <c r="G50" s="1" t="s">
         <v>68</v>
@@ -1603,7 +1690,7 @@
       <c r="N50" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="O50" s="10">
+      <c r="O50" s="10" t="n">
         <v>2</v>
       </c>
       <c r="P50" s="10" t="s">
@@ -1616,14 +1703,14 @@
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11"/>
       <c r="N51" s="10"/>
       <c r="O51" s="10"/>
       <c r="P51" s="10"/>
       <c r="Q51" s="11"/>
     </row>
-    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
         <v>72</v>
       </c>
@@ -1645,7 +1732,7 @@
       <c r="Q52" s="4"/>
       <c r="R52" s="4"/>
     </row>
-    <row r="53" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
         <v>53</v>
       </c>
@@ -1654,15 +1741,15 @@
         <v>73</v>
       </c>
     </row>
-    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O54" s="10"/>
       <c r="Q54" s="11"/>
     </row>
-    <row r="55" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="N55" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="O55" s="10">
+      <c r="O55" s="10" t="n">
         <v>1</v>
       </c>
       <c r="P55" s="10" t="s">
@@ -1673,11 +1760,11 @@
       </c>
       <c r="R55" s="10"/>
     </row>
-    <row r="56" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O56" s="11"/>
       <c r="Q56" s="11"/>
     </row>
-    <row r="57" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="3" t="s">
         <v>77</v>
       </c>
@@ -1701,12 +1788,12 @@
       </c>
       <c r="R57" s="4"/>
     </row>
-    <row r="58" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="59" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F59" s="1" t="s">
         <v>28</v>
       </c>
@@ -1716,14 +1803,14 @@
       <c r="N59" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O59" s="14">
-        <v>17.316948400000001</v>
+      <c r="O59" s="14" t="n">
+        <v>17.3169484</v>
       </c>
       <c r="P59" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F60" s="1" t="s">
         <v>30</v>
       </c>
@@ -1733,11 +1820,11 @@
       <c r="N60" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O60" s="14">
+      <c r="O60" s="14" t="n">
         <v>17.150216</v>
       </c>
     </row>
-    <row r="61" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F61" s="1" t="s">
         <v>31</v>
       </c>
@@ -1747,11 +1834,11 @@
       <c r="N61" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O61" s="14">
-        <v>17.411437070000002</v>
-      </c>
-    </row>
-    <row r="62" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O61" s="14" t="n">
+        <v>17.41143707</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F62" s="1" t="s">
         <v>32</v>
       </c>
@@ -1761,11 +1848,11 @@
       <c r="N62" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O62" s="14">
-        <v>18.210023199999998</v>
-      </c>
-    </row>
-    <row r="63" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O62" s="14" t="n">
+        <v>18.2100232</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F63" s="1" t="s">
         <v>34</v>
       </c>
@@ -1775,11 +1862,11 @@
       <c r="N63" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O63" s="14">
-        <v>19.589487999999999</v>
-      </c>
-    </row>
-    <row r="64" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O63" s="14" t="n">
+        <v>19.589488</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F64" s="1" t="s">
         <v>35</v>
       </c>
@@ -1789,11 +1876,11 @@
       <c r="N64" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O64" s="14">
+      <c r="O64" s="14" t="n">
         <v>19.4920008</v>
       </c>
     </row>
-    <row r="65" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F65" s="1" t="s">
         <v>36</v>
       </c>
@@ -1803,14 +1890,14 @@
       <c r="N65" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O65" s="14">
-        <v>18.194123999999999</v>
-      </c>
-    </row>
-    <row r="66" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O65" s="14" t="n">
+        <v>18.194124</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O66" s="14"/>
     </row>
-    <row r="67" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F67" s="1" t="s">
         <v>28</v>
       </c>
@@ -1820,11 +1907,11 @@
       <c r="N67" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O67" s="16">
+      <c r="O67" s="16" t="n">
         <v>7.55</v>
       </c>
     </row>
-    <row r="68" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F68" s="1" t="s">
         <v>30</v>
       </c>
@@ -1834,11 +1921,11 @@
       <c r="N68" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O68" s="16">
+      <c r="O68" s="16" t="n">
         <v>7.8</v>
       </c>
     </row>
-    <row r="69" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F69" s="1" t="s">
         <v>31</v>
       </c>
@@ -1848,11 +1935,11 @@
       <c r="N69" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O69" s="16">
-        <v>6.5666666669999998</v>
-      </c>
-    </row>
-    <row r="70" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O69" s="16" t="n">
+        <v>6.566666667</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F70" s="1" t="s">
         <v>32</v>
       </c>
@@ -1862,11 +1949,11 @@
       <c r="N70" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O70" s="16">
+      <c r="O70" s="16" t="n">
         <v>1.8</v>
       </c>
     </row>
-    <row r="71" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F71" s="1" t="s">
         <v>34</v>
       </c>
@@ -1876,11 +1963,11 @@
       <c r="N71" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O71" s="16">
+      <c r="O71" s="16" t="n">
         <v>7.15</v>
       </c>
     </row>
-    <row r="72" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F72" s="1" t="s">
         <v>35</v>
       </c>
@@ -1890,11 +1977,11 @@
       <c r="N72" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O72" s="16">
+      <c r="O72" s="16" t="n">
         <v>7.7</v>
       </c>
     </row>
-    <row r="73" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F73" s="1" t="s">
         <v>36</v>
       </c>
@@ -1904,14 +1991,14 @@
       <c r="N73" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O73" s="16">
+      <c r="O73" s="16" t="n">
         <v>5.9</v>
       </c>
     </row>
-    <row r="74" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O74" s="16"/>
     </row>
-    <row r="75" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F75" s="1" t="s">
         <v>28</v>
       </c>
@@ -1921,11 +2008,11 @@
       <c r="N75" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O75" s="16">
-        <v>2.4239999999999999</v>
-      </c>
-    </row>
-    <row r="76" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O75" s="16" t="n">
+        <v>2.424</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F76" s="1" t="s">
         <v>30</v>
       </c>
@@ -1935,11 +2022,11 @@
       <c r="N76" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O76" s="16">
-        <v>2.1280000000000001</v>
-      </c>
-    </row>
-    <row r="77" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O76" s="16" t="n">
+        <v>2.128</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F77" s="1" t="s">
         <v>31</v>
       </c>
@@ -1949,11 +2036,11 @@
       <c r="N77" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O77" s="16">
+      <c r="O77" s="16" t="n">
         <v>2.246666667</v>
       </c>
     </row>
-    <row r="78" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F78" s="1" t="s">
         <v>32</v>
       </c>
@@ -1963,11 +2050,11 @@
       <c r="N78" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O78" s="16">
-        <v>1.9359999999999999</v>
-      </c>
-    </row>
-    <row r="79" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O78" s="16" t="n">
+        <v>1.936</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F79" s="1" t="s">
         <v>34</v>
       </c>
@@ -1977,11 +2064,11 @@
       <c r="N79" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O79" s="16">
-        <v>8.2080000000000002</v>
-      </c>
-    </row>
-    <row r="80" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O79" s="16" t="n">
+        <v>8.208</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F80" s="1" t="s">
         <v>35</v>
       </c>
@@ -1991,11 +2078,11 @@
       <c r="N80" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O80" s="16">
-        <v>6.1520000000000001</v>
-      </c>
-    </row>
-    <row r="81" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O80" s="16" t="n">
+        <v>6.152</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F81" s="1" t="s">
         <v>36</v>
       </c>
@@ -2005,14 +2092,14 @@
       <c r="N81" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O81" s="16">
+      <c r="O81" s="16" t="n">
         <v>2.64</v>
       </c>
     </row>
-    <row r="82" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O82" s="16"/>
     </row>
-    <row r="83" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F83" s="1" t="s">
         <v>28</v>
       </c>
@@ -2022,11 +2109,11 @@
       <c r="N83" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O83" s="16">
-        <v>0.28000000000000003</v>
-      </c>
-    </row>
-    <row r="84" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O83" s="16" t="n">
+        <v>0.28</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F84" s="1" t="s">
         <v>30</v>
       </c>
@@ -2036,11 +2123,11 @@
       <c r="N84" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O84" s="16">
+      <c r="O84" s="16" t="n">
         <v>0.27</v>
       </c>
     </row>
-    <row r="85" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F85" s="1" t="s">
         <v>31</v>
       </c>
@@ -2050,11 +2137,11 @@
       <c r="N85" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O85" s="16">
+      <c r="O85" s="16" t="n">
         <v>0.27</v>
       </c>
     </row>
-    <row r="86" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F86" s="1" t="s">
         <v>32</v>
       </c>
@@ -2064,11 +2151,11 @@
       <c r="N86" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O86" s="16">
-        <v>0.34499999999999997</v>
-      </c>
-    </row>
-    <row r="87" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O86" s="16" t="n">
+        <v>0.345</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F87" s="1" t="s">
         <v>34</v>
       </c>
@@ -2078,11 +2165,11 @@
       <c r="N87" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O87" s="16">
-        <v>0.71499999999999997</v>
-      </c>
-    </row>
-    <row r="88" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O87" s="16" t="n">
+        <v>0.715</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F88" s="1" t="s">
         <v>35</v>
       </c>
@@ -2092,11 +2179,11 @@
       <c r="N88" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O88" s="16">
-        <v>1.2450000000000001</v>
-      </c>
-    </row>
-    <row r="89" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O88" s="16" t="n">
+        <v>1.245</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F89" s="1" t="s">
         <v>36</v>
       </c>
@@ -2106,14 +2193,14 @@
       <c r="N89" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O89" s="16">
-        <v>1.1950000000000001</v>
-      </c>
-    </row>
-    <row r="90" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O89" s="16" t="n">
+        <v>1.195</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O90" s="16"/>
     </row>
-    <row r="91" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F91" s="1" t="s">
         <v>28</v>
       </c>
@@ -2123,11 +2210,11 @@
       <c r="N91" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O91" s="16">
-        <v>2.4249999999999998</v>
-      </c>
-    </row>
-    <row r="92" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O91" s="16" t="n">
+        <v>2.425</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F92" s="1" t="s">
         <v>30</v>
       </c>
@@ -2137,11 +2224,11 @@
       <c r="N92" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O92" s="16">
+      <c r="O92" s="16" t="n">
         <v>2.34</v>
       </c>
     </row>
-    <row r="93" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F93" s="1" t="s">
         <v>31</v>
       </c>
@@ -2151,11 +2238,11 @@
       <c r="N93" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O93" s="16">
+      <c r="O93" s="16" t="n">
         <v>2.34</v>
       </c>
     </row>
-    <row r="94" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F94" s="1" t="s">
         <v>32</v>
       </c>
@@ -2165,11 +2252,11 @@
       <c r="N94" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O94" s="16">
-        <v>0.52500000000000002</v>
-      </c>
-    </row>
-    <row r="95" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="O94" s="16" t="n">
+        <v>0.525</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F95" s="1" t="s">
         <v>34</v>
       </c>
@@ -2179,11 +2266,11 @@
       <c r="N95" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O95" s="16">
+      <c r="O95" s="16" t="n">
         <v>2.35</v>
       </c>
     </row>
-    <row r="96" spans="6:15" x14ac:dyDescent="0.25">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F96" s="1" t="s">
         <v>35</v>
       </c>
@@ -2193,11 +2280,11 @@
       <c r="N96" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O96" s="16">
+      <c r="O96" s="16" t="n">
         <v>1.55</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F97" s="1" t="s">
         <v>36</v>
       </c>
@@ -2207,20 +2294,20 @@
       <c r="N97" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O97" s="16">
+      <c r="O97" s="16" t="n">
         <v>1.35</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O98" s="14"/>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="8" t="s">
         <v>87</v>
       </c>
       <c r="O99" s="14"/>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
         <v>53</v>
       </c>
@@ -2233,7 +2320,7 @@
       <c r="N100" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O100" s="14">
+      <c r="O100" s="14" t="n">
         <v>11.3</v>
       </c>
       <c r="P100" s="1" t="s">
@@ -2243,7 +2330,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
         <v>53</v>
       </c>
@@ -2256,12 +2343,12 @@
       <c r="N101" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O101" s="14">
+      <c r="O101" s="14" t="n">
         <v>10.1</v>
       </c>
       <c r="Q101" s="10"/>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
         <v>53</v>
       </c>
@@ -2274,12 +2361,12 @@
       <c r="N102" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O102" s="14">
-        <v>9.9416666669999998</v>
+      <c r="O102" s="14" t="n">
+        <v>9.941666667</v>
       </c>
       <c r="Q102" s="10"/>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
         <v>53</v>
       </c>
@@ -2292,12 +2379,12 @@
       <c r="N103" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O103" s="14">
+      <c r="O103" s="14" t="n">
         <v>14.1</v>
       </c>
       <c r="Q103" s="10"/>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
         <v>53</v>
       </c>
@@ -2310,12 +2397,12 @@
       <c r="N104" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O104" s="14">
+      <c r="O104" s="14" t="n">
         <v>14.6</v>
       </c>
       <c r="Q104" s="10"/>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
         <v>53</v>
       </c>
@@ -2328,12 +2415,12 @@
       <c r="N105" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O105" s="14">
+      <c r="O105" s="14" t="n">
         <v>12.2</v>
       </c>
       <c r="Q105" s="10"/>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
         <v>53</v>
       </c>
@@ -2346,16 +2433,16 @@
       <c r="N106" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O106" s="14">
+      <c r="O106" s="14" t="n">
         <v>11</v>
       </c>
       <c r="Q106" s="10"/>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O107" s="17"/>
       <c r="Q107" s="10"/>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
         <v>53</v>
       </c>
@@ -2368,7 +2455,7 @@
       <c r="N108" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O108" s="14">
+      <c r="O108" s="14" t="n">
         <v>13.35</v>
       </c>
       <c r="P108" s="1" t="s">
@@ -2376,7 +2463,7 @@
       </c>
       <c r="Q108" s="11"/>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
         <v>53</v>
       </c>
@@ -2389,12 +2476,12 @@
       <c r="N109" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O109" s="14">
+      <c r="O109" s="14" t="n">
         <v>11.9</v>
       </c>
       <c r="Q109" s="11"/>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
         <v>53</v>
       </c>
@@ -2407,12 +2494,12 @@
       <c r="N110" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O110" s="14">
+      <c r="O110" s="14" t="n">
         <v>12.4</v>
       </c>
       <c r="Q110" s="11"/>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="s">
         <v>53</v>
       </c>
@@ -2425,12 +2512,12 @@
       <c r="N111" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O111" s="14">
+      <c r="O111" s="14" t="n">
         <v>16</v>
       </c>
       <c r="Q111" s="11"/>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
         <v>53</v>
       </c>
@@ -2443,12 +2530,12 @@
       <c r="N112" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O112" s="14">
+      <c r="O112" s="14" t="n">
         <v>17.8</v>
       </c>
       <c r="Q112" s="11"/>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
         <v>53</v>
       </c>
@@ -2461,12 +2548,12 @@
       <c r="N113" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O113" s="14">
+      <c r="O113" s="14" t="n">
         <v>14.6</v>
       </c>
       <c r="Q113" s="11"/>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
         <v>53</v>
       </c>
@@ -2479,16 +2566,16 @@
       <c r="N114" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O114" s="14">
+      <c r="O114" s="14" t="n">
         <v>12.7</v>
       </c>
       <c r="Q114" s="11"/>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O115" s="17"/>
       <c r="Q115" s="11"/>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="s">
         <v>53</v>
       </c>
@@ -2501,7 +2588,7 @@
       <c r="N116" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O116" s="14">
+      <c r="O116" s="14" t="n">
         <v>20</v>
       </c>
       <c r="P116" s="1" t="s">
@@ -2511,7 +2598,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="s">
         <v>53</v>
       </c>
@@ -2524,12 +2611,12 @@
       <c r="N117" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O117" s="14">
+      <c r="O117" s="14" t="n">
         <v>20</v>
       </c>
       <c r="Q117" s="10"/>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="s">
         <v>53</v>
       </c>
@@ -2542,12 +2629,12 @@
       <c r="N118" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O118" s="14">
+      <c r="O118" s="14" t="n">
         <v>20</v>
       </c>
       <c r="Q118" s="11"/>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
         <v>53</v>
       </c>
@@ -2560,11 +2647,11 @@
       <c r="N119" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O119" s="14">
+      <c r="O119" s="14" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
         <v>53</v>
       </c>
@@ -2577,12 +2664,12 @@
       <c r="N120" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O120" s="14">
+      <c r="O120" s="14" t="n">
         <v>10</v>
       </c>
       <c r="Q120" s="10"/>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
         <v>53</v>
       </c>
@@ -2595,12 +2682,12 @@
       <c r="N121" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O121" s="14">
+      <c r="O121" s="14" t="n">
         <v>46</v>
       </c>
       <c r="Q121" s="11"/>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="1" t="s">
         <v>53</v>
       </c>
@@ -2613,15 +2700,15 @@
       <c r="N122" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O122" s="14">
+      <c r="O122" s="14" t="n">
         <v>45</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="O123" s="10"/>
       <c r="Q123" s="10"/>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="1" t="s">
         <v>53</v>
       </c>
@@ -2634,7 +2721,7 @@
       <c r="N124" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O124" s="14">
+      <c r="O124" s="14" t="n">
         <v>72</v>
       </c>
       <c r="P124" s="1" t="s">
@@ -2642,7 +2729,7 @@
       </c>
       <c r="Q124" s="11"/>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="1" t="s">
         <v>53</v>
       </c>
@@ -2656,14 +2743,14 @@
       <c r="N125" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O125" s="14">
+      <c r="O125" s="14" t="n">
         <v>69</v>
       </c>
       <c r="P125" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="1" t="s">
         <v>53</v>
       </c>
@@ -2676,7 +2763,7 @@
       <c r="N126" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O126" s="14">
+      <c r="O126" s="14" t="n">
         <v>74.3333333333333</v>
       </c>
       <c r="P126" s="1" t="s">
@@ -2684,7 +2771,7 @@
       </c>
       <c r="Q126" s="10"/>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="1" t="s">
         <v>53</v>
       </c>
@@ -2697,14 +2784,14 @@
       <c r="N127" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O127" s="14">
+      <c r="O127" s="14" t="n">
         <v>95</v>
       </c>
       <c r="P127" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="1" t="s">
         <v>53</v>
       </c>
@@ -2717,14 +2804,14 @@
       <c r="N128" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O128" s="14">
+      <c r="O128" s="14" t="n">
         <v>182</v>
       </c>
       <c r="P128" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="1" t="s">
         <v>53</v>
       </c>
@@ -2737,14 +2824,14 @@
       <c r="N129" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O129" s="14">
+      <c r="O129" s="14" t="n">
         <v>221</v>
       </c>
       <c r="P129" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="1" t="s">
         <v>53</v>
       </c>
@@ -2757,14 +2844,14 @@
       <c r="N130" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O130" s="14">
+      <c r="O130" s="14" t="n">
         <v>73</v>
       </c>
       <c r="P130" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="1" t="s">
         <v>53</v>
       </c>
@@ -2777,14 +2864,14 @@
       <c r="N132" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O132">
+      <c r="O132" s="1" t="n">
         <v>26.5</v>
       </c>
       <c r="P132" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="1" t="s">
         <v>53</v>
       </c>
@@ -2797,14 +2884,14 @@
       <c r="N133" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O133">
+      <c r="O133" s="1" t="n">
         <v>14</v>
       </c>
       <c r="P133" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="1" t="s">
         <v>53</v>
       </c>
@@ -2817,14 +2904,14 @@
       <c r="N134" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O134">
+      <c r="O134" s="1" t="n">
         <v>12.25</v>
       </c>
       <c r="P134" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="1" t="s">
         <v>53</v>
       </c>
@@ -2837,14 +2924,14 @@
       <c r="N135" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O135">
+      <c r="O135" s="1" t="n">
         <v>-33</v>
       </c>
       <c r="P135" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="1" t="s">
         <v>53</v>
       </c>
@@ -2857,14 +2944,14 @@
       <c r="N136" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O136">
+      <c r="O136" s="1" t="n">
         <v>261</v>
       </c>
       <c r="P136" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="1" t="s">
         <v>53</v>
       </c>
@@ -2877,14 +2964,14 @@
       <c r="N137" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O137">
+      <c r="O137" s="1" t="n">
         <v>79</v>
       </c>
       <c r="P137" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="1" t="s">
         <v>53</v>
       </c>
@@ -2897,15 +2984,42 @@
       <c r="N138" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O138">
+      <c r="O138" s="1" t="n">
         <v>36</v>
       </c>
       <c r="P138" s="1" t="s">
         <v>99</v>
       </c>
     </row>
+    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O141" s="1" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O142" s="1" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O144" s="1" t="n">
+        <f aca="false">O141*O108*22</f>
+        <v>234.96</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="O145" s="1" t="n">
+        <f aca="false">22*O142*O111</f>
+        <v>70.4</v>
+      </c>
+    </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>